<commit_message>
Add a tailored outreach message for each prospect
Hebrew message per business on the web page (with a name field and copy
button) and as a new column in the spreadsheet.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JAaRkUS1vckqNFGY4d1RtT
</commit_message>
<xml_diff>
--- a/research/Perko_Local_Business_Prospects_Jerusalem.xlsx
+++ b/research/Perko_Local_Business_Prospects_Jerusalem.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$3:$W$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$3:$X$23</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -563,7 +563,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W23"/>
+  <dimension ref="A1:X23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -589,6 +589,7 @@
     <col width="12" customWidth="1" min="21" max="21"/>
     <col width="14" customWidth="1" min="22" max="22"/>
     <col width="44" customWidth="1" min="23" max="23"/>
+    <col width="60" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -619,6 +620,7 @@
       <c r="U1" s="2" t="n"/>
       <c r="V1" s="2" t="n"/>
       <c r="W1" s="2" t="n"/>
+      <c r="X1" s="2" t="n"/>
     </row>
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
@@ -648,6 +650,7 @@
       <c r="U2" s="2" t="n"/>
       <c r="V2" s="2" t="n"/>
       <c r="W2" s="2" t="n"/>
+      <c r="X2" s="2" t="n"/>
     </row>
     <row r="3" ht="36" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
@@ -765,6 +768,11 @@
           <t>Additional Notes</t>
         </is>
       </c>
+      <c r="X3" s="4" t="inlineStr">
+        <is>
+          <t>Suggested Outreach Message (Hebrew)</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="96" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
@@ -874,6 +882,16 @@
       <c r="W4" s="6" t="inlineStr">
         <is>
           <t>Phone confirmed on the official site (2026-10-25). Street number 20 from rest.co.il (https://www.rest.co.il/rest/80358238/) and Debbest; the official site gives no number. Founders named on own site and in Times of Israel FR (Aug 2023). No email published.</t>
+        </is>
+      </c>
+      <c r="X4" s="5" t="inlineStr">
+        <is>
+          <t>היי מיכאל ודניאל,
+אני [השם שלך] מ-Perko. ראיתי מה בניתם בבירמה: קלייה קטנה, דלפק עם לקוחות קבועים שעוצרים בדרך לעבודה. בדיוק העסק שכרטיס חותמות נועד בשבילו.
+אנחנו מפתחים כרטיס נאמנות דיגיטלי משותף לעסקים בשכונה. במקום כרטיס נייר, הלקוח סורק קוד בקופה וצובר חותמות לפי הכללים שלכם, והכרטיס שלכם יושב באותה אפליקציה עם עוד עסקים מהרחוב.
+אנחנו בגישה מוקדמת ומחפשים כמה עסקים ראשונים שיעזרו לנו לבנות את זה נכון. ההצטרפות כרגע בחינם, בלי התחייבות.
+בא לכם 15 דקות שיחה השבוע? אשמח להגיע לדלפק.
+[השם שלך]</t>
         </is>
       </c>
     </row>
@@ -983,6 +1001,17 @@
           <t>Email and phone confirmed on the official contact page (2026-10-25). Single location; company פרידה קאלו בע"מ. Owner not named publicly. Directory hours conflict, so check before visiting.</t>
         </is>
       </c>
+      <c r="X5" s="9" t="inlineStr">
+        <is>
+          <t>שלום לצוות קאלו,
+אני [השם שלך] מ-Perko. קאלו הוא כבר שנים חלק מהשגרה של בקעה, גם בבית הקפה וגם במעדנייה, ונראה לי שיש לכם בדיוק את הקהל הקבוע שאנחנו בונים בשבילו.
+Perko הוא כרטיס נאמנות דיגיטלי משותף לעסקים בשכונה: הלקוח סורק קוד בקופה, צובר חותמות או נקודות לפי ההטבה שאתם מגדירים, ורואה באותה אפליקציה גם עסקים נוספים בדרך בית לחם.
+אנחנו בשלב גישה מוקדמת ומחפשים עסקים ראשונים שישפיעו על איך המוצר יעבוד בקופה. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום.
+אשמח לדבר עם מי שאחראי אצלכם על הלקוחות, או לקפוץ ולהראות. למי כדאי לפנות?
+תודה,
+[השם שלך]</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="96" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
@@ -1098,6 +1127,17 @@
           <t>Email and phone confirmed on the official About page (2026-10-25). Listed at no. 23 in The Jerusalem Guide German Colony feature (3 Jul 2026). Social URLs taken from the official site. Emek Refaim light-rail works may affect footfall in 2026.</t>
         </is>
       </c>
+      <c r="X6" s="5" t="inlineStr">
+        <is>
+          <t>שלום לאה ואבי,
+אני [השם שלך] מ-Perko. טחנת הקפה היא מקום שאנשים חוזרים אליו כל בוקר, וגם קונים שוב את הפולים שלכם כל כמה שבועות.
+אנחנו בונים כרטיס נאמנות דיגיטלי משותף לעסקים בשכונה: הלקוח סורק קוד בקופה, צובר חותמות לפי הכללים שאתם קובעים, ורואה באותה אפליקציה גם כרטיסים של עסקים אחרים ברחוב.
+אנחנו בשלב גישה מוקדמת ומחפשים כמה עסקים ראשונים בעמק רפאים שיעזרו לנו לעצב את המוצר. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום.
+אשמח ל-15 דקות שיחה או לקפץ אליכם לקפה ולהראות במה מדובר. מתי נוח לכם?
+תודה,
+[השם שלך]</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="96" customHeight="1">
       <c r="A7" s="9" t="inlineStr">
@@ -1203,6 +1243,16 @@
       <c r="W7" s="10" t="inlineStr">
         <is>
           <t>Official site (webflow) checked 2026-10-25: Instagram link present, no phone. Phones conflict across directories: rest.co.il 058-4296540, Google (via Wanderlog) 02-631-0295. Google reviews dated Dec 2025 and Jan 2026 per Wanderlog. casalavicafe.com did not load (TLS error).</t>
+        </is>
+      </c>
+      <c r="X7" s="9" t="inlineStr">
+        <is>
+          <t>היי מיטל ואלפונסו,
+אני [השם שלך] מ-Perko. אהבתי את מה שבניתם בקאסה לביא: קלייה משלכם, מאפים בריאים, וקהל שחוזר כמה פעמים בשבוע.
+אנחנו מפתחים כרטיס נאמנות דיגיטלי משותף לעסקים בשכונה. הלקוח סורק קוד בקופה, צובר חותמות לפי הכללים שלכם, ורואה באותה אפליקציה גם עסקים שכנים בדרך בית לחם.
+אנחנו בגישה מוקדמת ומחפשים כמה עסקים ראשונים שיעזרו לנו לעצב את המוצר. ההצטרפות כרגע בחינם, בלי התחייבות.
+אשמח לקפוץ לקפה ולהראות בכמה דקות. מתי נוח לכם?
+[השם שלך]</t>
         </is>
       </c>
     </row>
@@ -1300,6 +1350,16 @@
           <t>Phone confirmed on the official site (2026-10-25); site footer ©2026 with current hours (Sun-Thu 10-19, Fri 7-16). Owner not named. A Wolt listing was seen in search results only.</t>
         </is>
       </c>
+      <c r="X8" s="5" t="inlineStr">
+        <is>
+          <t>שלום לצוות פרחי העמק,
+אני [השם שלך] מ-Perko. הרבה משפחות בשכונה קונות פרחים לשבת כל שבוע, וזה בדיוק סוג הקנייה החוזרת שאנחנו בונים בשבילו.
+Perko הוא כרטיס נאמנות דיגיטלי משותף לעסקים ברחוב: הלקוח סורק קוד בקופה וצובר חותמות לפי מה שאתם מחליטים, למשל זר תשיעי במתנה. באותה אפליקציה הוא רואה גם בתי קפה ועסקים אחרים בעמק רפאים.
+אנחנו בגישה מוקדמת ומחפשים עסקים ראשונים. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום.
+אשמח לשיחה של 10 דקות או לקפוץ לחנות. מתי מתאים?
+[השם שלך]</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="96" customHeight="1">
       <c r="A9" s="9" t="inlineStr">
@@ -1395,6 +1455,16 @@
           <t>Wolt listing live (open on 25 Oct 2026). A second number, +972-54-522-2843, appears on Wolt. History from Hebrew Wikipedia's Derech Beit Lehem article. No website or published email.</t>
         </is>
       </c>
+      <c r="X9" s="9" t="inlineStr">
+        <is>
+          <t>היי, שלום לצוות של המקום של איציק,
+אני [השם שלך] מ-Perko. אתם מהמקומות שהשכונה חוזרת אליהם כל יום, עוד מימי הקיוסק.
+אנחנו בונים כרטיס נאמנות דיגיטלי משותף לעסקים בדרך בית לחם. בלי כרטיס נייר ובלי אפליקציה נפרדת: הלקוח סורק קוד בקופה, צובר חותמות לפי מה שתחליטו (למשל קפה עשירי חינם), ובאותה אפליקציה רואה גם עסקים שכנים.
+אנחנו בגישה מוקדמת ומחפשים כמה עסקים ראשונים ברחוב. ההצטרפות כרגע בחינם, בלי התחייבות, ואנחנו עושים את כל ההקמה.
+אפשר לקפוץ אליכם לכמה דקות בשעה שקטה ולהראות? מה הזמן הכי נוח?
+[השם שלך]</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="96" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
@@ -1492,6 +1562,17 @@
       <c r="W10" s="6" t="inlineStr">
         <is>
           <t>Phone confirmed on the official site (2026-10-25). Live on Wolt. One search snippet mentioned further branches (HaNasi St, Herzl Blvd), but neither the official site nor a Mako article lists them, so independence is not fully confirmed. Seasonal demand (summer peak).</t>
+        </is>
+      </c>
+      <c r="X10" s="5" t="inlineStr">
+        <is>
+          <t>שלום לצוות ציגה,
+אני [השם שלך] מ-Perko. גלידה היא בדיוק הדבר שמשפחות מהשכונה חוזרות אליו שוב ושוב, ולכן חשבנו עליכם.
+Perko הוא כרטיס נאמנות דיגיטלי משותף לעסקים בשכונה: הלקוח סורק קוד בקופה וצובר חותמות לפי ההטבה שאתם קובעים, למשל ״כל כדור שמיני עלינו״. הכרטיס שלכם יופיע באותה אפליקציה עם עסקים נוספים בדרך בית לחם.
+אנחנו בגישה מוקדמת ומחפשים עסקים ראשונים שיעזרו לנו לבנות את המוצר. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום.
+אשמח לשיחה קצרה או לקפוץ אליכם. מתי נוח?
+תודה,
+[השם שלך]</t>
         </is>
       </c>
     </row>
@@ -1589,6 +1670,16 @@
           <t>Live on Wolt (rating 9.2; open 25 Oct 2026). The Facebook page is the 'website' listed on Wolt. An Instagram handle @bresaola.jlm was seen only in search results, so it is not included. The domain bresaola-jerusalem.com did not resolve.</t>
         </is>
       </c>
+      <c r="X11" s="9" t="inlineStr">
+        <is>
+          <t>שלום לצוות ברזאולה,
+אני [השם שלך] מ-Perko. יש לכם קהל מעריצים אמיתי, ומגיעים אליכם גם לקניות הביתה וגם לערב בבר.
+אנחנו בונים כרטיס נאמנות דיגיטלי משותף לעסקים בשכונה: הלקוח סורק קוד בקופה וצובר חותמות לפי ההטבה שאתם קובעים, ובאותה אפליקציה רואה גם עסקים שכנים בדרך בית לחם.
+אנחנו בגישה מוקדמת ומחפשים עסקים ראשונים שיעזרו לנו לבנות את המוצר. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום.
+אשמח לקפוץ אליכם לכמה דקות. מתי הכי שקט אצלכם?
+[השם שלך]</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="96" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
@@ -1690,6 +1781,17 @@
       <c r="W12" s="6" t="inlineStr">
         <is>
           <t>Email and phone confirmed on the official site (2026-10-25). The Wolt URL suffix '-emek-refaim' might hint at other branches, but none was found. Two florists on Emek Refaim (with Emek Flowers) may compete, so pitch them separately.</t>
+        </is>
+      </c>
+      <c r="X12" s="5" t="inlineStr">
+        <is>
+          <t>שלום לצוות הפרחים של ארז,
+אני [השם שלך] מ-Perko. יש לכם גם קונים שנכנסים לחנות לפני שבת וגם לקוחות משלוחים שחוזרים, וזה בדיוק הקהל שאנחנו בונים בשבילו.
+Perko הוא כרטיס נאמנות דיגיטלי משותף לעסקים בעמק רפאים: הלקוח סורק קוד בקופה וצובר חותמות לפי ההטבה שאתם מגדירים, ובאותה אפליקציה רואה גם עסקים נוספים ברחוב.
+אנחנו בשלב גישה מוקדמת ומחפשים עסקים ראשונים. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום.
+אשמח לשיחה של 10 דקות. מתי נוח לכם?
+תודה,
+[השם שלך]</t>
         </is>
       </c>
     </row>
@@ -1791,6 +1893,17 @@
           <t>Email and phone confirmed on the official site (2026-10-25); Sukkot 2026 promotions live. Directories show other numbers (d.co.il 077-3164751), so use the official one.</t>
         </is>
       </c>
+      <c r="X13" s="9" t="inlineStr">
+        <is>
+          <t>שלום לצוות פלורה,
+אני [השם שלך] מ-Perko. פרחים לשבת, ועוד שיאים בחגים, הם בדיוק סוג הקנייה החוזרת שאנחנו בונים בשבילו.
+Perko הוא כרטיס נאמנות דיגיטלי משותף לעסקים בשכונה: הלקוח סורק קוד בקופה וצובר חותמות לפי מה שאתם מחליטים, למשל זר תשיעי במתנה. באותה אפליקציה הוא רואה גם בתי קפה ועסקים שכנים בדרך בית לחם.
+אנחנו בשלב גישה מוקדמת ומחפשים כמה עסקים ראשונים. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום.
+אשמח לשיחה קצרה או לקפוץ לחנות. מתי נוח לכם?
+תודה,
+[השם שלך]</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="96" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
@@ -1900,6 +2013,17 @@
       <c r="W14" s="6" t="inlineStr">
         <is>
           <t>Phone, WhatsApp and Instagram confirmed on the official site (2026-10-25). Live on Wolt. No email published (events contact form only).</t>
+        </is>
+      </c>
+      <c r="X14" s="5" t="inlineStr">
+        <is>
+          <t>שלום עדי ושרה,
+אני [השם שלך] מ-Perko. גראנד קפה הוא אחד המקומות שמגדירים את בקעה, עם קהל בראנץ' נאמן.
+אנחנו בונים כרטיס נאמנות דיגיטלי משותף לעסקים בשכונה: הלקוח סורק קוד בקופה וצובר חותמות או נקודות לפי ההטבה שאתם מגדירים, למשל מאפה עלינו בביקור באמצע השבוע. באותה אפליקציה הוא רואה גם עסקים נוספים בדרך בית לחם.
+אנחנו בגישה מוקדמת ומחפשים עסקים ראשונים שיעזרו לנו לבנות את זה. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום.
+אשמח לפגישה קצרה בזמן שנוח לכם. מתי מתאים?
+תודה,
+[השם שלך]</t>
         </is>
       </c>
     </row>
@@ -1999,6 +2123,16 @@
       <c r="W15" s="10" t="inlineStr">
         <is>
           <t>Phone confirmed on the official site (2026-10-25). Wolt lists 02-6444966. A Mazav article (Jun 2021) names three Jerusalem restaurateurs as owners who also run other restaurants: a single shop, but not a lone owner. Names left out because the source is from 2021.</t>
+        </is>
+      </c>
+      <c r="X15" s="9" t="inlineStr">
+        <is>
+          <t>שלום לצוות לה שרולה,
+אני [השם שלך] מ-Perko. הרבה משפחות בשכונה קונות אצלכם בשר לשבת כל שבוע, וזה בדיוק סוג הלקוח הקבוע שאנחנו בונים בשבילו.
+Perko הוא כרטיס נאמנות דיגיטלי משותף לעסקים בשכונה: הלקוח סורק קוד בקופה וצובר נקודות לפי הכללים שלכם, והכרטיס שלכם יושב באותה אפליקציה עם עסקים נוספים בדרך בית לחם.
+אנחנו בגישה מוקדמת ומחפשים עסקים ראשונים. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום.
+אשמח לשיחה קצרה עם מי שמנהל את החנות. מתי נוח?
+[השם שלך]</t>
         </is>
       </c>
     </row>
@@ -2092,6 +2226,16 @@
           <t>Score reduced because current operation is not firmly verified: rest.co.il updated Feb 2026 and listed in iTravelJerusalem, but no dated 2026 review was found. Confirm it is open before outreach. Shares no. 35 with Focaccia Moshava.</t>
         </is>
       </c>
+      <c r="X16" s="5" t="inlineStr">
+        <is>
+          <t>שלום לצוות לחם ועוד,
+אני [השם שלך] מ-Perko. מאפייה היא המקום שאנשים חוזרים אליו הכי הרבה, ללחם של כל יום ולעוגות של שבת.
+אנחנו בונים כרטיס נאמנות דיגיטלי משותף לעסקים בעמק רפאים: הלקוח סורק קוד בקופה, צובר חותמות לפי ההטבה שאתם קובעים, ורואה באותה אפליקציה גם עסקים שכנים ברחוב.
+אנחנו בגישה מוקדמת ומחפשים עסקים ראשונים. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום.
+אשמח לקפוץ ולהראות בכמה דקות. מתי מתאים?
+[השם שלך]</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="96" customHeight="1">
       <c r="A17" s="9" t="inlineStr">
@@ -2195,6 +2339,16 @@
           <t>Small local family group (also runs two Buchman pizza places), not a chain. Wolt listing seen in search results. Kashrut wording differs between sources. No 2026-dated evidence found.</t>
         </is>
       </c>
+      <c r="X17" s="9" t="inlineStr">
+        <is>
+          <t>היי ליאור ומתן,
+אני [השם שלך] מ-Perko. הדיינר שלכם הוא מקום שמשפחות ובני נוער חוזרים אליו, וזה בדיוק הקהל שכרטיס חותמות עובד אצלו הכי טוב.
+Perko הוא כרטיס נאמנות דיגיטלי משותף לעסקים בשכונה: הלקוח סורק קוד בקופה וצובר חותמות לפי ההטבה שאתם קובעים, למשל מילקשייק חינם בביקור השישי. באותה אפליקציה הוא רואה גם עסקים נוספים בעמק רפאים.
+אנחנו בגישה מוקדמת ומחפשים עסקים ראשונים. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום, ואם זה יעבוד אפשר יהיה להרחיב גם למקומות הנוספים שלכם.
+אשמח לשיחה קצרה. מתי נוח?
+[השם שלך]</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="96" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
@@ -2300,6 +2454,16 @@
       <c r="W18" s="6" t="inlineStr">
         <is>
           <t>Phone and Instagram confirmed on the official site after rendering it (2026-10-25). Afternoon tea is more of an occasion than a daily visit. Hebrew Wikipedia names a different owner; the 2026 Times of Israel article was used instead. GoKosher lists another phone, 077-5373226.</t>
+        </is>
+      </c>
+      <c r="X18" s="5" t="inlineStr">
+        <is>
+          <t>שלום אלישבע,
+אני [השם שלך] מ-Perko. קראתי עלייך ועל קומקום, ואהבתי את הבית הקטן והקהילתי שבנית בבקעה.
+אנחנו מפתחים כרטיס נאמנות דיגיטלי משותף לעסקים בשכונה: הלקוח סורק קוד בקופה וצובר חותמות לפי מה שתבחרי, למשל קנקן תה או סקונס במתנה, וגם קניות של תה עלים לבית נספרות. באותה אפליקציה הוא רואה גם עסקים שכנים בדרך בית לחם.
+אנחנו בגישה מוקדמת ומחפשים עסקים ראשונים. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום.
+אשמח לבוא לתה ולהראות בכמה דקות. מתי נוח לך?
+[השם שלך]</t>
         </is>
       </c>
     </row>
@@ -2393,6 +2557,17 @@
           <t>Kosher sibling of the downtown Focaccia Bar (Rabbi Akiva St): a local two-location brand, not a single independent shop. Listed in The Jerusalem Guide (3 Jul 2026). A website (m.focaccia.co) appears on iTravelJerusalem but was not verified, so it is left blank.</t>
         </is>
       </c>
+      <c r="X19" s="9" t="inlineStr">
+        <is>
+          <t>שלום לצוות פוקצ'ה במושבה,
+אני [השם שלך] מ-Perko. שוק הפוקצ'ות שלכם בשישי הוא בדיוק הרגל שבועי שכדאי לתגמל.
+אנחנו בונים כרטיס נאמנות דיגיטלי משותף לעסקים בעמק רפאים: הלקוח סורק קוד בקופה וצובר חותמות לפי ההטבה שאתם קובעים, למשל פוקצ'ה עלינו בשישי העשירי. באותה אפליקציה הוא רואה גם עסקים שכנים ברחוב.
+אנחנו בגישה מוקדמת ומחפשים עסקים ראשונים. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום.
+אשמח לדבר עם מי שמנהל את הסניף. מתי נוח?
+תודה,
+[השם שלך]</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="96" customHeight="1">
       <c r="A20" s="5" t="inlineStr">
@@ -2484,6 +2659,17 @@
           <t>Listed in The Jerusalem Guide German Colony feature (3 Jul 2026). No official site or social profile found. The latest rest.co.il review is from 2023.</t>
         </is>
       </c>
+      <c r="X20" s="5" t="inlineStr">
+        <is>
+          <t>שלום לצוות פומפידו,
+אני [השם שלך] מ-Perko. אנחנו בונים כרטיס נאמנות דיגיטלי משותף לעסקים בעמק רפאים: הלקוח סורק קוד בקופה וצובר נקודות לפי ההטבה שאתם קובעים, למשל קינוח עלינו בביקור הרביעי.
+היתרון בשבילכם הוא החיבור לעסקים השכנים: לקוחות שמכירים את הרחוב מבתי הקפה ביום יכולים לגלות אתכם בערב דרך אותה אפליקציה.
+אנחנו בגישה מוקדמת ומחפשים עסקים ראשונים. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום.
+אשמח לדבר עם מי שמנהל את המקום. מתי אפשר לתפוס אתכם?
+תודה,
+[השם שלך]</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="96" customHeight="1">
       <c r="A21" s="9" t="inlineStr">
@@ -2575,6 +2761,16 @@
           <t>rest.co.il updated Jun 2026 with a user review dated 19 Aug 2025 (negative). Sources disagree on the cuisine label. The 074 number may be a directory routing number; confirm the direct line in person. Farther from the central cluster.</t>
         </is>
       </c>
+      <c r="X21" s="9" t="inlineStr">
+        <is>
+          <t>שלום לצוות רנדבו,
+אני [השם שלך] מ-Perko. פיצה ופסטה הן הזמנות שמשפחות חוזרות אליהן שוב ושוב, וזה בדיוק המקום שבו כרטיס חותמות עובד.
+Perko הוא כרטיס נאמנות דיגיטלי משותף לעסקים בדרך בית לחם: הלקוח סורק קוד בקופה וצובר חותמות לפי ההטבה שאתם קובעים, ובאותה אפליקציה רואה גם עסקים נוספים ברחוב.
+אנחנו בגישה מוקדמת ומחפשים עסקים ראשונים. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום.
+אשמח לשיחה קצרה עם מי שמנהל את המקום. מתי נוח?
+[השם שלך]</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="96" customHeight="1">
       <c r="A22" s="5" t="inlineStr">
@@ -2674,6 +2870,17 @@
           <t>Email and phone confirmed on the official contact page (2026-10-25). Local brand with two of its own shops (Emek Refaim 6 and Shlomtzion St), not a chain. The contact page lists first names (Barbara, Boaz) without roles, so no contact person is recorded. No 2025-26 dated evidence found.</t>
         </is>
       </c>
+      <c r="X22" s="5" t="inlineStr">
+        <is>
+          <t>שלום ברברה,
+אני [השם שלך] מ-Perko. אנחנו בונים כרטיס נאמנות דיגיטלי משותף לעסקים בעמק רפאים: הלקוח סורק קוד בקופה, צובר הטבות לפי הכללים של כל עסק, ורואה באותה אפליקציה את כל העסקים המשתתפים ברחוב.
+בשביל חנות מתנות היתרון העיקרי הוא החשיפה: לקוחות קבועים של בתי הקפה והמאפיות ברחוב יכולים לגלות אתכם, במיוחד לפני החגים. ההטבה יכולה להיות משהו קטן, כמו עטיפת מתנה או הנחה לקנייה הבאה.
+אנחנו בגישה מוקדמת. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום.
+אשמח לשמוע אם זה מעניין אותך.
+תודה,
+[השם שלך]</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="96" customHeight="1">
       <c r="A23" s="9" t="inlineStr">
@@ -2789,9 +2996,20 @@
           <t>Email and phone confirmed on the official site (2026-10-25); footer © 2026. Low purchase frequency, so better as a later-phase partner than a pilot anchor.</t>
         </is>
       </c>
+      <c r="X23" s="9" t="inlineStr">
+        <is>
+          <t>שלום דליה ואייל,
+אני [השם שלך] מ-Perko. סתיו תכשיטים הוא מהעסקים הוותיקים והמיוחדים בעמק רפאים, וזה בדיוק סוג המקום שאנחנו רוצים שאנשים מהשכונה יגלו.
+אנחנו בונים כרטיס נאמנות דיגיטלי משותף לעסקים ברחוב. אצלכם זה לא יהיה כרטיס חותמות רגיל: אפשר להגדיר הטבה שמתאימה לתכשיטים, כמו ניקוי, תיקון או חריטה במתנה, ולהגיע ללקוחות של בתי הקפה והחנויות השכנות באותה אפליקציה.
+אנחנו בגישה מוקדמת. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום.
+אשמח לשמוע אם זה מעניין אתכם, ולקפוץ לשיחה קצרה.
+תודה,
+[השם שלך]</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:W23"/>
+  <autoFilter ref="A3:X23"/>
   <conditionalFormatting sqref="P4:P23">
     <cfRule type="cellIs" priority="1" operator="greaterThanOrEqual" dxfId="0">
       <formula>8</formula>

</xml_diff>

<commit_message>
Add small-business and community paragraph to all outreach messages
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JAaRkUS1vckqNFGY4d1RtT
</commit_message>
<xml_diff>
--- a/research/Perko_Local_Business_Prospects_Jerusalem.xlsx
+++ b/research/Perko_Local_Business_Prospects_Jerusalem.xlsx
@@ -889,6 +889,7 @@
           <t>היי מיכאל ודניאל,
 אני [השם שלך] מ-Perko. ראיתי מה בניתם בבירמה: קלייה קטנה, דלפק עם לקוחות קבועים שעוצרים בדרך לעבודה. בדיוק העסק שכרטיס חותמות נועד בשבילו.
 אנחנו מפתחים כרטיס נאמנות דיגיטלי משותף לעסקים בשכונה. במקום כרטיס נייר, הלקוח סורק קוד בקופה וצובר חותמות לפי הכללים שלכם, והכרטיס שלכם יושב באותה אפליקציה עם עוד עסקים מהרחוב.
+פרקו נולדה כדי לשמור על העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כל ניקוב בכרטיס הוא עוד סיבה לחזור לעסק המקומי ולחזק את הקהילה שסביבו.
 אנחנו בגישה מוקדמת ומחפשים כמה עסקים ראשונים שיעזרו לנו לבנות את זה נכון. ההצטרפות כרגע בחינם, בלי התחייבות.
 בא לכם 15 דקות שיחה השבוע? אשמח להגיע לדלפק.
 [השם שלך]</t>
@@ -1006,6 +1007,7 @@
           <t>שלום לצוות קאלו,
 אני [השם שלך] מ-Perko. קאלו הוא כבר שנים חלק מהשגרה של בקעה, גם בבית הקפה וגם במעדנייה, ונראה לי שיש לכם בדיוק את הקהל הקבוע שאנחנו בונים בשבילו.
 Perko הוא כרטיס נאמנות דיגיטלי משותף לעסקים בשכונה: הלקוח סורק קוד בקופה, צובר חותמות או נקודות לפי ההטבה שאתם מגדירים, ורואה באותה אפליקציה גם עסקים נוספים בדרך בית לחם.
+פרקו נולדה כדי לשמור על העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כל ניקוב בכרטיס הוא עוד סיבה לחזור לעסק המקומי ולחזק את הקהילה שסביבו.
 אנחנו בשלב גישה מוקדמת ומחפשים עסקים ראשונים שישפיעו על איך המוצר יעבוד בקופה. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום.
 אשמח לדבר עם מי שאחראי אצלכם על הלקוחות, או לקפוץ ולהראות. למי כדאי לפנות?
 תודה,
@@ -1132,6 +1134,7 @@
           <t>שלום לאה ואבי,
 אני [השם שלך] מ-Perko. טחנת הקפה היא מקום שאנשים חוזרים אליו כל בוקר, וגם קונים שוב את הפולים שלכם כל כמה שבועות.
 אנחנו בונים כרטיס נאמנות דיגיטלי משותף לעסקים בשכונה: הלקוח סורק קוד בקופה, צובר חותמות לפי הכללים שאתם קובעים, ורואה באותה אפליקציה גם כרטיסים של עסקים אחרים ברחוב.
+פרקו נולדה כדי לשמור על העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כל ניקוב בכרטיס הוא עוד סיבה לחזור לעסק המקומי ולחזק את הקהילה שסביבו.
 אנחנו בשלב גישה מוקדמת ומחפשים כמה עסקים ראשונים בעמק רפאים שיעזרו לנו לעצב את המוצר. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום.
 אשמח ל-15 דקות שיחה או לקפץ אליכם לקפה ולהראות במה מדובר. מתי נוח לכם?
 תודה,
@@ -1250,6 +1253,7 @@
           <t>היי מיטל ואלפונסו,
 אני [השם שלך] מ-Perko. אהבתי את מה שבניתם בקאסה לביא: קלייה משלכם, מאפים בריאים, וקהל שחוזר כמה פעמים בשבוע.
 אנחנו מפתחים כרטיס נאמנות דיגיטלי משותף לעסקים בשכונה. הלקוח סורק קוד בקופה, צובר חותמות לפי הכללים שלכם, ורואה באותה אפליקציה גם עסקים שכנים בדרך בית לחם.
+פרקו נולדה כדי לשמור על העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כל ניקוב בכרטיס הוא עוד סיבה לחזור לעסק המקומי ולחזק את הקהילה שסביבו.
 אנחנו בגישה מוקדמת ומחפשים כמה עסקים ראשונים שיעזרו לנו לעצב את המוצר. ההצטרפות כרגע בחינם, בלי התחייבות.
 אשמח לקפוץ לקפה ולהראות בכמה דקות. מתי נוח לכם?
 [השם שלך]</t>
@@ -1355,6 +1359,7 @@
           <t>שלום לצוות פרחי העמק,
 אני [השם שלך] מ-Perko. הרבה משפחות בשכונה קונות פרחים לשבת כל שבוע, וזה בדיוק סוג הקנייה החוזרת שאנחנו בונים בשבילו.
 Perko הוא כרטיס נאמנות דיגיטלי משותף לעסקים ברחוב: הלקוח סורק קוד בקופה וצובר חותמות לפי מה שאתם מחליטים, למשל זר תשיעי במתנה. באותה אפליקציה הוא רואה גם בתי קפה ועסקים אחרים בעמק רפאים.
+פרקו נולדה כדי לשמור על העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כל ניקוב בכרטיס הוא עוד סיבה לחזור לעסק המקומי ולחזק את הקהילה שסביבו.
 אנחנו בגישה מוקדמת ומחפשים עסקים ראשונים. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום.
 אשמח לשיחה של 10 דקות או לקפוץ לחנות. מתי מתאים?
 [השם שלך]</t>
@@ -1460,6 +1465,7 @@
           <t>היי, שלום לצוות של המקום של איציק,
 אני [השם שלך] מ-Perko. אתם מהמקומות שהשכונה חוזרת אליהם כל יום, עוד מימי הקיוסק.
 אנחנו בונים כרטיס נאמנות דיגיטלי משותף לעסקים בדרך בית לחם. בלי כרטיס נייר ובלי אפליקציה נפרדת: הלקוח סורק קוד בקופה, צובר חותמות לפי מה שתחליטו (למשל קפה עשירי חינם), ובאותה אפליקציה רואה גם עסקים שכנים.
+פרקו נולדה כדי לשמור על העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כל ניקוב בכרטיס הוא עוד סיבה לחזור לעסק המקומי ולחזק את הקהילה שסביבו.
 אנחנו בגישה מוקדמת ומחפשים כמה עסקים ראשונים ברחוב. ההצטרפות כרגע בחינם, בלי התחייבות, ואנחנו עושים את כל ההקמה.
 אפשר לקפוץ אליכם לכמה דקות בשעה שקטה ולהראות? מה הזמן הכי נוח?
 [השם שלך]</t>
@@ -1569,6 +1575,7 @@
           <t>שלום לצוות ציגה,
 אני [השם שלך] מ-Perko. גלידה היא בדיוק הדבר שמשפחות מהשכונה חוזרות אליו שוב ושוב, ולכן חשבנו עליכם.
 Perko הוא כרטיס נאמנות דיגיטלי משותף לעסקים בשכונה: הלקוח סורק קוד בקופה וצובר חותמות לפי ההטבה שאתם קובעים, למשל ״כל כדור שמיני עלינו״. הכרטיס שלכם יופיע באותה אפליקציה עם עסקים נוספים בדרך בית לחם.
+פרקו נולדה כדי לשמור על העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כל ניקוב בכרטיס הוא עוד סיבה לחזור לעסק המקומי ולחזק את הקהילה שסביבו.
 אנחנו בגישה מוקדמת ומחפשים עסקים ראשונים שיעזרו לנו לבנות את המוצר. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום.
 אשמח לשיחה קצרה או לקפוץ אליכם. מתי נוח?
 תודה,
@@ -1675,6 +1682,7 @@
           <t>שלום לצוות ברזאולה,
 אני [השם שלך] מ-Perko. יש לכם קהל מעריצים אמיתי, ומגיעים אליכם גם לקניות הביתה וגם לערב בבר.
 אנחנו בונים כרטיס נאמנות דיגיטלי משותף לעסקים בשכונה: הלקוח סורק קוד בקופה וצובר חותמות לפי ההטבה שאתם קובעים, ובאותה אפליקציה רואה גם עסקים שכנים בדרך בית לחם.
+פרקו נולדה כדי לשמור על העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כל ניקוב בכרטיס הוא עוד סיבה לחזור לעסק המקומי ולחזק את הקהילה שסביבו.
 אנחנו בגישה מוקדמת ומחפשים עסקים ראשונים שיעזרו לנו לבנות את המוצר. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום.
 אשמח לקפוץ אליכם לכמה דקות. מתי הכי שקט אצלכם?
 [השם שלך]</t>
@@ -1788,6 +1796,7 @@
           <t>שלום לצוות הפרחים של ארז,
 אני [השם שלך] מ-Perko. יש לכם גם קונים שנכנסים לחנות לפני שבת וגם לקוחות משלוחים שחוזרים, וזה בדיוק הקהל שאנחנו בונים בשבילו.
 Perko הוא כרטיס נאמנות דיגיטלי משותף לעסקים בעמק רפאים: הלקוח סורק קוד בקופה וצובר חותמות לפי ההטבה שאתם מגדירים, ובאותה אפליקציה רואה גם עסקים נוספים ברחוב.
+פרקו נולדה כדי לשמור על העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כל ניקוב בכרטיס הוא עוד סיבה לחזור לעסק המקומי ולחזק את הקהילה שסביבו.
 אנחנו בשלב גישה מוקדמת ומחפשים עסקים ראשונים. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום.
 אשמח לשיחה של 10 דקות. מתי נוח לכם?
 תודה,
@@ -1898,6 +1907,7 @@
           <t>שלום לצוות פלורה,
 אני [השם שלך] מ-Perko. פרחים לשבת, ועוד שיאים בחגים, הם בדיוק סוג הקנייה החוזרת שאנחנו בונים בשבילו.
 Perko הוא כרטיס נאמנות דיגיטלי משותף לעסקים בשכונה: הלקוח סורק קוד בקופה וצובר חותמות לפי מה שאתם מחליטים, למשל זר תשיעי במתנה. באותה אפליקציה הוא רואה גם בתי קפה ועסקים שכנים בדרך בית לחם.
+פרקו נולדה כדי לשמור על העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כל ניקוב בכרטיס הוא עוד סיבה לחזור לעסק המקומי ולחזק את הקהילה שסביבו.
 אנחנו בשלב גישה מוקדמת ומחפשים כמה עסקים ראשונים. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום.
 אשמח לשיחה קצרה או לקפוץ לחנות. מתי נוח לכם?
 תודה,
@@ -2020,6 +2030,7 @@
           <t>שלום עדי ושרה,
 אני [השם שלך] מ-Perko. גראנד קפה הוא אחד המקומות שמגדירים את בקעה, עם קהל בראנץ' נאמן.
 אנחנו בונים כרטיס נאמנות דיגיטלי משותף לעסקים בשכונה: הלקוח סורק קוד בקופה וצובר חותמות או נקודות לפי ההטבה שאתם מגדירים, למשל מאפה עלינו בביקור באמצע השבוע. באותה אפליקציה הוא רואה גם עסקים נוספים בדרך בית לחם.
+פרקו נולדה כדי לשמור על העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כל ניקוב בכרטיס הוא עוד סיבה לחזור לעסק המקומי ולחזק את הקהילה שסביבו.
 אנחנו בגישה מוקדמת ומחפשים עסקים ראשונים שיעזרו לנו לבנות את זה. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום.
 אשמח לפגישה קצרה בזמן שנוח לכם. מתי מתאים?
 תודה,
@@ -2130,6 +2141,7 @@
           <t>שלום לצוות לה שרולה,
 אני [השם שלך] מ-Perko. הרבה משפחות בשכונה קונות אצלכם בשר לשבת כל שבוע, וזה בדיוק סוג הלקוח הקבוע שאנחנו בונים בשבילו.
 Perko הוא כרטיס נאמנות דיגיטלי משותף לעסקים בשכונה: הלקוח סורק קוד בקופה וצובר נקודות לפי הכללים שלכם, והכרטיס שלכם יושב באותה אפליקציה עם עסקים נוספים בדרך בית לחם.
+פרקו נולדה כדי לשמור על העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כל ניקוב בכרטיס הוא עוד סיבה לחזור לעסק המקומי ולחזק את הקהילה שסביבו.
 אנחנו בגישה מוקדמת ומחפשים עסקים ראשונים. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום.
 אשמח לשיחה קצרה עם מי שמנהל את החנות. מתי נוח?
 [השם שלך]</t>
@@ -2231,6 +2243,7 @@
           <t>שלום לצוות לחם ועוד,
 אני [השם שלך] מ-Perko. מאפייה היא המקום שאנשים חוזרים אליו הכי הרבה, ללחם של כל יום ולעוגות של שבת.
 אנחנו בונים כרטיס נאמנות דיגיטלי משותף לעסקים בעמק רפאים: הלקוח סורק קוד בקופה, צובר חותמות לפי ההטבה שאתם קובעים, ורואה באותה אפליקציה גם עסקים שכנים ברחוב.
+פרקו נולדה כדי לשמור על העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כל ניקוב בכרטיס הוא עוד סיבה לחזור לעסק המקומי ולחזק את הקהילה שסביבו.
 אנחנו בגישה מוקדמת ומחפשים עסקים ראשונים. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום.
 אשמח לקפוץ ולהראות בכמה דקות. מתי מתאים?
 [השם שלך]</t>
@@ -2344,6 +2357,7 @@
           <t>היי ליאור ומתן,
 אני [השם שלך] מ-Perko. הדיינר שלכם הוא מקום שמשפחות ובני נוער חוזרים אליו, וזה בדיוק הקהל שכרטיס חותמות עובד אצלו הכי טוב.
 Perko הוא כרטיס נאמנות דיגיטלי משותף לעסקים בשכונה: הלקוח סורק קוד בקופה וצובר חותמות לפי ההטבה שאתם קובעים, למשל מילקשייק חינם בביקור השישי. באותה אפליקציה הוא רואה גם עסקים נוספים בעמק רפאים.
+פרקו נולדה כדי לשמור על העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כל ניקוב בכרטיס הוא עוד סיבה לחזור לעסק המקומי ולחזק את הקהילה שסביבו.
 אנחנו בגישה מוקדמת ומחפשים עסקים ראשונים. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום, ואם זה יעבוד אפשר יהיה להרחיב גם למקומות הנוספים שלכם.
 אשמח לשיחה קצרה. מתי נוח?
 [השם שלך]</t>
@@ -2461,6 +2475,7 @@
           <t>שלום אלישבע,
 אני [השם שלך] מ-Perko. קראתי עלייך ועל קומקום, ואהבתי את הבית הקטן והקהילתי שבנית בבקעה.
 אנחנו מפתחים כרטיס נאמנות דיגיטלי משותף לעסקים בשכונה: הלקוח סורק קוד בקופה וצובר חותמות לפי מה שתבחרי, למשל קנקן תה או סקונס במתנה, וגם קניות של תה עלים לבית נספרות. באותה אפליקציה הוא רואה גם עסקים שכנים בדרך בית לחם.
+פרקו נולדה כדי לשמור על העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כל ניקוב בכרטיס הוא עוד סיבה לחזור לעסק המקומי ולחזק את הקהילה שסביבו.
 אנחנו בגישה מוקדמת ומחפשים עסקים ראשונים. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום.
 אשמח לבוא לתה ולהראות בכמה דקות. מתי נוח לך?
 [השם שלך]</t>
@@ -2562,6 +2577,7 @@
           <t>שלום לצוות פוקצ'ה במושבה,
 אני [השם שלך] מ-Perko. שוק הפוקצ'ות שלכם בשישי הוא בדיוק הרגל שבועי שכדאי לתגמל.
 אנחנו בונים כרטיס נאמנות דיגיטלי משותף לעסקים בעמק רפאים: הלקוח סורק קוד בקופה וצובר חותמות לפי ההטבה שאתם קובעים, למשל פוקצ'ה עלינו בשישי העשירי. באותה אפליקציה הוא רואה גם עסקים שכנים ברחוב.
+פרקו נולדה כדי לשמור על העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כל ניקוב בכרטיס הוא עוד סיבה לחזור לעסק המקומי ולחזק את הקהילה שסביבו.
 אנחנו בגישה מוקדמת ומחפשים עסקים ראשונים. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום.
 אשמח לדבר עם מי שמנהל את הסניף. מתי נוח?
 תודה,
@@ -2664,6 +2680,7 @@
           <t>שלום לצוות פומפידו,
 אני [השם שלך] מ-Perko. אנחנו בונים כרטיס נאמנות דיגיטלי משותף לעסקים בעמק רפאים: הלקוח סורק קוד בקופה וצובר נקודות לפי ההטבה שאתם קובעים, למשל קינוח עלינו בביקור הרביעי.
 היתרון בשבילכם הוא החיבור לעסקים השכנים: לקוחות שמכירים את הרחוב מבתי הקפה ביום יכולים לגלות אתכם בערב דרך אותה אפליקציה.
+פרקו נולדה כדי לשמור על העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כל ניקוב בכרטיס הוא עוד סיבה לחזור לעסק המקומי ולחזק את הקהילה שסביבו.
 אנחנו בגישה מוקדמת ומחפשים עסקים ראשונים. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום.
 אשמח לדבר עם מי שמנהל את המקום. מתי אפשר לתפוס אתכם?
 תודה,
@@ -2766,6 +2783,7 @@
           <t>שלום לצוות רנדבו,
 אני [השם שלך] מ-Perko. פיצה ופסטה הן הזמנות שמשפחות חוזרות אליהן שוב ושוב, וזה בדיוק המקום שבו כרטיס חותמות עובד.
 Perko הוא כרטיס נאמנות דיגיטלי משותף לעסקים בדרך בית לחם: הלקוח סורק קוד בקופה וצובר חותמות לפי ההטבה שאתם קובעים, ובאותה אפליקציה רואה גם עסקים נוספים ברחוב.
+פרקו נולדה כדי לשמור על העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כל ניקוב בכרטיס הוא עוד סיבה לחזור לעסק המקומי ולחזק את הקהילה שסביבו.
 אנחנו בגישה מוקדמת ומחפשים עסקים ראשונים. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום.
 אשמח לשיחה קצרה עם מי שמנהל את המקום. מתי נוח?
 [השם שלך]</t>
@@ -2875,6 +2893,7 @@
           <t>שלום ברברה,
 אני [השם שלך] מ-Perko. אנחנו בונים כרטיס נאמנות דיגיטלי משותף לעסקים בעמק רפאים: הלקוח סורק קוד בקופה, צובר הטבות לפי הכללים של כל עסק, ורואה באותה אפליקציה את כל העסקים המשתתפים ברחוב.
 בשביל חנות מתנות היתרון העיקרי הוא החשיפה: לקוחות קבועים של בתי הקפה והמאפיות ברחוב יכולים לגלות אתכם, במיוחד לפני החגים. ההטבה יכולה להיות משהו קטן, כמו עטיפת מתנה או הנחה לקנייה הבאה.
+פרקו נולדה כדי לשמור על העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כל ניקוב בכרטיס הוא עוד סיבה לחזור לעסק המקומי ולחזק את הקהילה שסביבו.
 אנחנו בגישה מוקדמת. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום.
 אשמח לשמוע אם זה מעניין אותך.
 תודה,
@@ -3001,6 +3020,7 @@
           <t>שלום דליה ואייל,
 אני [השם שלך] מ-Perko. סתיו תכשיטים הוא מהעסקים הוותיקים והמיוחדים בעמק רפאים, וזה בדיוק סוג המקום שאנחנו רוצים שאנשים מהשכונה יגלו.
 אנחנו בונים כרטיס נאמנות דיגיטלי משותף לעסקים ברחוב. אצלכם זה לא יהיה כרטיס חותמות רגיל: אפשר להגדיר הטבה שמתאימה לתכשיטים, כמו ניקוי, תיקון או חריטה במתנה, ולהגיע ללקוחות של בתי הקפה והחנויות השכנות באותה אפליקציה.
+פרקו נולדה כדי לשמור על העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כל ניקוב בכרטיס הוא עוד סיבה לחזור לעסק המקומי ולחזק את הקהילה שסביבו.
 אנחנו בגישה מוקדמת. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום.
 אשמח לשמוע אם זה מעניין אתכם, ולקפוץ לשיחה קצרה.
 תודה,

</xml_diff>

<commit_message>
Research: rewrite the 20 outreach messages and add a clean HTML prospect sheet
Shorter, warmer messages (same honesty rules: early access, free, no claims
that anyone joined). New research/perko-outreach.html, Excel and JSON synced.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VZAuLHaESUH9foWg6jPqbt
</commit_message>
<xml_diff>
--- a/research/Perko_Local_Business_Prospects_Jerusalem.xlsx
+++ b/research/Perko_Local_Business_Prospects_Jerusalem.xlsx
@@ -887,11 +887,10 @@
       <c r="X4" s="5" t="inlineStr">
         <is>
           <t>היי מיכאל ודניאל,
-אני [השם שלך] מ-Perko. ראיתי מה בניתם בבירמה: קלייה קטנה, דלפק עם לקוחות קבועים שעוצרים בדרך לעבודה. בדיוק העסק שכרטיס חותמות נועד בשבילו.
-אנחנו מפתחים כרטיס נאמנות דיגיטלי משותף לעסקים בשכונה. במקום כרטיס נייר, הלקוח סורק קוד בקופה וצובר חותמות לפי הכללים שלכם, והכרטיס שלכם יושב באותה אפליקציה עם עוד עסקים מהרחוב.
-פרקו נולדה כדי לשמור על העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כל ניקוב בכרטיס הוא עוד סיבה לחזור לעסק המקומי ולחזק את הקהילה שסביבו.
-אנחנו בגישה מוקדמת ומחפשים כמה עסקים ראשונים שיעזרו לנו לבנות את זה נכון. ההצטרפות כרגע בחינם, בלי התחייבות.
-בא לכם 15 דקות שיחה השבוע? אשמח להגיע לדלפק.
+כאן [השם שלך] מפרקו. בירמה היא בדיוק סוג המקום שאנחנו בונים בשבילו: קלייה קטנה ודלפק עם לקוחות קבועים שעוצרים בדרך לעבודה.
+פרקו מחליפה את כרטיס הנייר באפליקציה אחת לכל העסקים בשכונה. הלקוח סורק קוד בקופה, צובר חותמות לפי הכללים שלכם, ורואה שם גם עסקים נוספים ברחוב.
+אנחנו רוצים לחזק את העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כרגע אנחנו בגישה מוקדמת, וההצטרפות בחינם ובלי התחייבות.
+יש לכם רבע שעה השבוע? אשמח להגיע לדלפק.
 [השם שלך]</t>
         </is>
       </c>
@@ -1005,11 +1004,10 @@
       <c r="X5" s="9" t="inlineStr">
         <is>
           <t>שלום לצוות קאלו,
-אני [השם שלך] מ-Perko. קאלו הוא כבר שנים חלק מהשגרה של בקעה, גם בבית הקפה וגם במעדנייה, ונראה לי שיש לכם בדיוק את הקהל הקבוע שאנחנו בונים בשבילו.
-Perko הוא כרטיס נאמנות דיגיטלי משותף לעסקים בשכונה: הלקוח סורק קוד בקופה, צובר חותמות או נקודות לפי ההטבה שאתם מגדירים, ורואה באותה אפליקציה גם עסקים נוספים בדרך בית לחם.
-פרקו נולדה כדי לשמור על העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כל ניקוב בכרטיס הוא עוד סיבה לחזור לעסק המקומי ולחזק את הקהילה שסביבו.
-אנחנו בשלב גישה מוקדמת ומחפשים עסקים ראשונים שישפיעו על איך המוצר יעבוד בקופה. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום.
-אשמח לדבר עם מי שאחראי אצלכם על הלקוחות, או לקפוץ ולהראות. למי כדאי לפנות?
+כאן [השם שלך] מפרקו. קאלו הוא כבר שנים חלק מהשגרה של בקעה, גם בבית הקפה וגם במעדנייה.
+פרקו היא אפליקציה אחת לכרטיסי מועדון של עסקים בשכונה. הלקוח סורק קוד בקופה וצובר חותמות לפי הכללים שלכם, למשל ארוחת בוקר עשירית עליכם. באותה אפליקציה הלקוח רואה גם עסקים נוספים בדרך בית לחם.
+אנחנו רוצים לחזק את העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כרגע אנחנו בגישה מוקדמת, וההצטרפות בחינם ובלי התחייבות.
+אשמח לדבר עם מי שאחראי אצלכם על הלקוחות. למי כדאי לפנות?
 תודה,
 [השם שלך]</t>
         </is>
@@ -1132,11 +1130,10 @@
       <c r="X6" s="5" t="inlineStr">
         <is>
           <t>שלום לאה ואבי,
-אני [השם שלך] מ-Perko. טחנת הקפה היא מקום שאנשים חוזרים אליו כל בוקר, וגם קונים שוב את הפולים שלכם כל כמה שבועות.
-אנחנו בונים כרטיס נאמנות דיגיטלי משותף לעסקים בשכונה: הלקוח סורק קוד בקופה, צובר חותמות לפי הכללים שאתם קובעים, ורואה באותה אפליקציה גם כרטיסים של עסקים אחרים ברחוב.
-פרקו נולדה כדי לשמור על העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כל ניקוב בכרטיס הוא עוד סיבה לחזור לעסק המקומי ולחזק את הקהילה שסביבו.
-אנחנו בשלב גישה מוקדמת ומחפשים כמה עסקים ראשונים בעמק רפאים שיעזרו לנו לעצב את המוצר. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום.
-אשמח ל-15 דקות שיחה או לקפץ אליכם לקפה ולהראות במה מדובר. מתי נוח לכם?
+כאן [השם שלך] מפרקו. טחנת הקפה היא מהמקומות שאנשים בעמק רפאים חוזרים אליהם כל בוקר, וגם לשקית הפולים כל כמה שבועות.
+פרקו היא אפליקציה אחת לכרטיסי מועדון של עסקים בשכונה. הלקוח סורק קוד בקופה וצובר חותמות לפי הכללים שלכם, למשל קפה עשירי עליכם או הנחה על שקית פולים.
+אנחנו רוצים לחזק את העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כרגע אנחנו בגישה מוקדמת, וההצטרפות בחינם ובלי התחייבות.
+אשמח לקפוץ לקפה ולהראות לכם את זה בעשר דקות. מתי נוח?
 תודה,
 [השם שלך]</t>
         </is>
@@ -1251,11 +1248,10 @@
       <c r="X7" s="9" t="inlineStr">
         <is>
           <t>היי מיטל ואלפונסו,
-אני [השם שלך] מ-Perko. אהבתי את מה שבניתם בקאסה לביא: קלייה משלכם, מאפים בריאים, וקהל שחוזר כמה פעמים בשבוע.
-אנחנו מפתחים כרטיס נאמנות דיגיטלי משותף לעסקים בשכונה. הלקוח סורק קוד בקופה, צובר חותמות לפי הכללים שלכם, ורואה באותה אפליקציה גם עסקים שכנים בדרך בית לחם.
-פרקו נולדה כדי לשמור על העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כל ניקוב בכרטיס הוא עוד סיבה לחזור לעסק המקומי ולחזק את הקהילה שסביבו.
-אנחנו בגישה מוקדמת ומחפשים כמה עסקים ראשונים שיעזרו לנו לעצב את המוצר. ההצטרפות כרגע בחינם, בלי התחייבות.
-אשמח לקפוץ לקפה ולהראות בכמה דקות. מתי נוח לכם?
+כאן [השם שלך] מפרקו. אהבנו את מה שבניתם בקאסה לביא: קלייה משלכם, מאפים בריאים וקהל שחוזר כמה פעמים בשבוע.
+פרקו היא אפליקציה אחת לכרטיסי מועדון של עסקים בשכונה. הלקוח סורק קוד בקופה וצובר חותמות לפי הכללים שלכם, ורואה שם גם עסקים שכנים בדרך בית לחם.
+אנחנו רוצים לחזק את העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כרגע אנחנו בגישה מוקדמת, וההצטרפות בחינם ובלי התחייבות.
+אשמח לקפוץ לקפה ולהראות את זה בכמה דקות. מתי נוח לכם?
 [השם שלך]</t>
         </is>
       </c>
@@ -1357,11 +1353,10 @@
       <c r="X8" s="5" t="inlineStr">
         <is>
           <t>שלום לצוות פרחי העמק,
-אני [השם שלך] מ-Perko. הרבה משפחות בשכונה קונות פרחים לשבת כל שבוע, וזה בדיוק סוג הקנייה החוזרת שאנחנו בונים בשבילו.
-Perko הוא כרטיס נאמנות דיגיטלי משותף לעסקים ברחוב: הלקוח סורק קוד בקופה וצובר חותמות לפי מה שאתם מחליטים, למשל זר תשיעי במתנה. באותה אפליקציה הוא רואה גם בתי קפה ועסקים אחרים בעמק רפאים.
-פרקו נולדה כדי לשמור על העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כל ניקוב בכרטיס הוא עוד סיבה לחזור לעסק המקומי ולחזק את הקהילה שסביבו.
-אנחנו בגישה מוקדמת ומחפשים עסקים ראשונים. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום.
-אשמח לשיחה של 10 דקות או לקפוץ לחנות. מתי מתאים?
+כאן [השם שלך] מפרקו. הרבה משפחות בשכונה קונות פרחים לשבת כל שבוע, וזה בדיוק הלקוח הקבוע שאנחנו בונים בשבילו.
+פרקו היא אפליקציה אחת לכרטיסי מועדון של עסקים בשכונה. הלקוח סורק קוד בקופה וצובר חותמות לפי הכללים שלכם, למשל זר תשיעי במתנה. באותה אפליקציה הוא רואה גם את בתי הקפה והחנויות השכנות בעמק רפאים.
+אנחנו רוצים לחזק את העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כרגע אנחנו בגישה מוקדמת, וההצטרפות בחינם ובלי התחייבות.
+אשמח לעשר דקות שיחה או לקפוץ לחנות. מתי מתאים?
 [השם שלך]</t>
         </is>
       </c>
@@ -1462,12 +1457,11 @@
       </c>
       <c r="X9" s="9" t="inlineStr">
         <is>
-          <t>היי, שלום לצוות של המקום של איציק,
-אני [השם שלך] מ-Perko. אתם מהמקומות שהשכונה חוזרת אליהם כל יום, עוד מימי הקיוסק.
-אנחנו בונים כרטיס נאמנות דיגיטלי משותף לעסקים בדרך בית לחם. בלי כרטיס נייר ובלי אפליקציה נפרדת: הלקוח סורק קוד בקופה, צובר חותמות לפי מה שתחליטו (למשל קפה עשירי חינם), ובאותה אפליקציה רואה גם עסקים שכנים.
-פרקו נולדה כדי לשמור על העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כל ניקוב בכרטיס הוא עוד סיבה לחזור לעסק המקומי ולחזק את הקהילה שסביבו.
-אנחנו בגישה מוקדמת ומחפשים כמה עסקים ראשונים ברחוב. ההצטרפות כרגע בחינם, בלי התחייבות, ואנחנו עושים את כל ההקמה.
-אפשר לקפוץ אליכם לכמה דקות בשעה שקטה ולהראות? מה הזמן הכי נוח?
+          <t>שלום לצוות של המקום של איציק,
+כאן [השם שלך] מפרקו. אתם מהמקומות שהשכונה חוזרת אליהם כל יום, עוד מימי הקיוסק.
+פרקו היא כרטיס מועדון דיגיטלי אחד לעסקים בדרך בית לחם, בלי כרטיס נייר ובלי אפליקציה נפרדת. הלקוח סורק קוד בקופה וצובר חותמות לפי מה שתחליטו, למשל קפה עשירי חינם.
+אנחנו רוצים לחזק את העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כרגע אנחנו בגישה מוקדמת, וההצטרפות בחינם ובלי התחייבות.
+אפשר לקפוץ אליכם לכמה דקות בשעה שקטה? מתי הכי נוח?
 [השם שלך]</t>
         </is>
       </c>
@@ -1573,10 +1567,9 @@
       <c r="X10" s="5" t="inlineStr">
         <is>
           <t>שלום לצוות ציגה,
-אני [השם שלך] מ-Perko. גלידה היא בדיוק הדבר שמשפחות מהשכונה חוזרות אליו שוב ושוב, ולכן חשבנו עליכם.
-Perko הוא כרטיס נאמנות דיגיטלי משותף לעסקים בשכונה: הלקוח סורק קוד בקופה וצובר חותמות לפי ההטבה שאתם קובעים, למשל ״כל כדור שמיני עלינו״. הכרטיס שלכם יופיע באותה אפליקציה עם עסקים נוספים בדרך בית לחם.
-פרקו נולדה כדי לשמור על העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כל ניקוב בכרטיס הוא עוד סיבה לחזור לעסק המקומי ולחזק את הקהילה שסביבו.
-אנחנו בגישה מוקדמת ומחפשים עסקים ראשונים שיעזרו לנו לבנות את המוצר. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום.
+כאן [השם שלך] מפרקו. גלידה היא בדיוק הפינוק שמשפחות מהשכונה חוזרות אליו שוב ושוב.
+פרקו היא אפליקציה אחת לכרטיסי מועדון של עסקים בשכונה. הלקוח סורק קוד בקופה וצובר חותמות לפי הכללים שלכם, למשל ״כל כדור שמיני עלינו״.
+אנחנו רוצים לחזק את העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כרגע אנחנו בגישה מוקדמת, וההצטרפות בחינם ובלי התחייבות.
 אשמח לשיחה קצרה או לקפוץ אליכם. מתי נוח?
 תודה,
 [השם שלך]</t>
@@ -1680,10 +1673,9 @@
       <c r="X11" s="9" t="inlineStr">
         <is>
           <t>שלום לצוות ברזאולה,
-אני [השם שלך] מ-Perko. יש לכם קהל מעריצים אמיתי, ומגיעים אליכם גם לקניות הביתה וגם לערב בבר.
-אנחנו בונים כרטיס נאמנות דיגיטלי משותף לעסקים בשכונה: הלקוח סורק קוד בקופה וצובר חותמות לפי ההטבה שאתם קובעים, ובאותה אפליקציה רואה גם עסקים שכנים בדרך בית לחם.
-פרקו נולדה כדי לשמור על העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כל ניקוב בכרטיס הוא עוד סיבה לחזור לעסק המקומי ולחזק את הקהילה שסביבו.
-אנחנו בגישה מוקדמת ומחפשים עסקים ראשונים שיעזרו לנו לבנות את המוצר. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום.
+כאן [השם שלך] מפרקו. יש לכם קהל נאמן אמיתי, שמגיע גם לקניות הביתה וגם לערב בבר.
+פרקו היא אפליקציה אחת לכרטיסי מועדון של עסקים בשכונה. הלקוח סורק קוד בקופה וצובר חותמות לפי הכללים שלכם, ורואה שם גם עסקים שכנים בדרך בית לחם.
+אנחנו רוצים לחזק את העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כרגע אנחנו בגישה מוקדמת, וההצטרפות בחינם ובלי התחייבות.
 אשמח לקפוץ אליכם לכמה דקות. מתי הכי שקט אצלכם?
 [השם שלך]</t>
         </is>
@@ -1794,11 +1786,10 @@
       <c r="X12" s="5" t="inlineStr">
         <is>
           <t>שלום לצוות הפרחים של ארז,
-אני [השם שלך] מ-Perko. יש לכם גם קונים שנכנסים לחנות לפני שבת וגם לקוחות משלוחים שחוזרים, וזה בדיוק הקהל שאנחנו בונים בשבילו.
-Perko הוא כרטיס נאמנות דיגיטלי משותף לעסקים בעמק רפאים: הלקוח סורק קוד בקופה וצובר חותמות לפי ההטבה שאתם מגדירים, ובאותה אפליקציה רואה גם עסקים נוספים ברחוב.
-פרקו נולדה כדי לשמור על העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כל ניקוב בכרטיס הוא עוד סיבה לחזור לעסק המקומי ולחזק את הקהילה שסביבו.
-אנחנו בשלב גישה מוקדמת ומחפשים עסקים ראשונים. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום.
-אשמח לשיחה של 10 דקות. מתי נוח לכם?
+כאן [השם שלך] מפרקו. יש לכם גם קונים שנכנסים לפני שבת וגם לקוחות משלוחים שחוזרים, וזה בדיוק הקהל שאנחנו בונים בשבילו.
+פרקו היא אפליקציה אחת לכרטיסי מועדון של עסקים בשכונה. הלקוח סורק קוד בקופה וצובר חותמות לפי הכללים שלכם, ורואה שם גם עסקים נוספים בעמק רפאים.
+אנחנו רוצים לחזק את העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כרגע אנחנו בגישה מוקדמת, וההצטרפות בחינם ובלי התחייבות.
+אשמח לעשר דקות שיחה. מתי נוח לכם?
 תודה,
 [השם שלך]</t>
         </is>
@@ -1905,10 +1896,9 @@
       <c r="X13" s="9" t="inlineStr">
         <is>
           <t>שלום לצוות פלורה,
-אני [השם שלך] מ-Perko. פרחים לשבת, ועוד שיאים בחגים, הם בדיוק סוג הקנייה החוזרת שאנחנו בונים בשבילו.
-Perko הוא כרטיס נאמנות דיגיטלי משותף לעסקים בשכונה: הלקוח סורק קוד בקופה וצובר חותמות לפי מה שאתם מחליטים, למשל זר תשיעי במתנה. באותה אפליקציה הוא רואה גם בתי קפה ועסקים שכנים בדרך בית לחם.
-פרקו נולדה כדי לשמור על העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כל ניקוב בכרטיס הוא עוד סיבה לחזור לעסק המקומי ולחזק את הקהילה שסביבו.
-אנחנו בשלב גישה מוקדמת ומחפשים כמה עסקים ראשונים. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום.
+כאן [השם שלך] מפרקו. פרחים לשבת ולחגים הם בדיוק קנייה שחוזרת על עצמה, ושווה לתגמל עליה.
+פרקו היא אפליקציה אחת לכרטיסי מועדון של עסקים בשכונה. הלקוח סורק קוד בקופה וצובר חותמות לפי הכללים שלכם, למשל זר תשיעי במתנה. באותה אפליקציה הוא רואה גם בתי קפה ועסקים שכנים בדרך בית לחם.
+אנחנו רוצים לחזק את העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כרגע אנחנו בגישה מוקדמת, וההצטרפות בחינם ובלי התחייבות.
 אשמח לשיחה קצרה או לקפוץ לחנות. מתי נוח לכם?
 תודה,
 [השם שלך]</t>
@@ -2028,11 +2018,10 @@
       <c r="X14" s="5" t="inlineStr">
         <is>
           <t>שלום עדי ושרה,
-אני [השם שלך] מ-Perko. גראנד קפה הוא אחד המקומות שמגדירים את בקעה, עם קהל בראנץ' נאמן.
-אנחנו בונים כרטיס נאמנות דיגיטלי משותף לעסקים בשכונה: הלקוח סורק קוד בקופה וצובר חותמות או נקודות לפי ההטבה שאתם מגדירים, למשל מאפה עלינו בביקור באמצע השבוע. באותה אפליקציה הוא רואה גם עסקים נוספים בדרך בית לחם.
-פרקו נולדה כדי לשמור על העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כל ניקוב בכרטיס הוא עוד סיבה לחזור לעסק המקומי ולחזק את הקהילה שסביבו.
-אנחנו בגישה מוקדמת ומחפשים עסקים ראשונים שיעזרו לנו לבנות את זה. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום.
-אשמח לפגישה קצרה בזמן שנוח לכם. מתי מתאים?
+כאן [השם שלך] מפרקו. גראנד קפה הוא מהמקומות שמגדירים את בקעה, עם קהל בראנץ' נאמן.
+פרקו היא אפליקציה אחת לכרטיסי מועדון של עסקים בשכונה. הלקוח סורק קוד בקופה וצובר חותמות לפי הכללים שלכם, למשל מאפה עליכם בביקור באמצע השבוע.
+אנחנו רוצים לחזק את העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כרגע אנחנו בגישה מוקדמת, וההצטרפות בחינם ובלי התחייבות.
+אשמח לפגישה קצרה בזמן שנוח לכם.
 תודה,
 [השם שלך]</t>
         </is>
@@ -2139,10 +2128,9 @@
       <c r="X15" s="9" t="inlineStr">
         <is>
           <t>שלום לצוות לה שרולה,
-אני [השם שלך] מ-Perko. הרבה משפחות בשכונה קונות אצלכם בשר לשבת כל שבוע, וזה בדיוק סוג הלקוח הקבוע שאנחנו בונים בשבילו.
-Perko הוא כרטיס נאמנות דיגיטלי משותף לעסקים בשכונה: הלקוח סורק קוד בקופה וצובר נקודות לפי הכללים שלכם, והכרטיס שלכם יושב באותה אפליקציה עם עסקים נוספים בדרך בית לחם.
-פרקו נולדה כדי לשמור על העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כל ניקוב בכרטיס הוא עוד סיבה לחזור לעסק המקומי ולחזק את הקהילה שסביבו.
-אנחנו בגישה מוקדמת ומחפשים עסקים ראשונים. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום.
+כאן [השם שלך] מפרקו. הרבה משפחות בשכונה קונות אצלכם לשבת כל שבוע, וזה בדיוק הלקוח הקבוע שאנחנו בונים בשבילו.
+פרקו היא אפליקציה אחת לכרטיסי מועדון של עסקים בשכונה. הלקוח סורק קוד בקופה וצובר נקודות לפי הכללים שלכם, ורואה שם גם עסקים נוספים בדרך בית לחם.
+אנחנו רוצים לחזק את העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כרגע אנחנו בגישה מוקדמת, וההצטרפות בחינם ובלי התחייבות.
 אשמח לשיחה קצרה עם מי שמנהל את החנות. מתי נוח?
 [השם שלך]</t>
         </is>
@@ -2241,11 +2229,10 @@
       <c r="X16" s="5" t="inlineStr">
         <is>
           <t>שלום לצוות לחם ועוד,
-אני [השם שלך] מ-Perko. מאפייה היא המקום שאנשים חוזרים אליו הכי הרבה, ללחם של כל יום ולעוגות של שבת.
-אנחנו בונים כרטיס נאמנות דיגיטלי משותף לעסקים בעמק רפאים: הלקוח סורק קוד בקופה, צובר חותמות לפי ההטבה שאתם קובעים, ורואה באותה אפליקציה גם עסקים שכנים ברחוב.
-פרקו נולדה כדי לשמור על העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כל ניקוב בכרטיס הוא עוד סיבה לחזור לעסק המקומי ולחזק את הקהילה שסביבו.
-אנחנו בגישה מוקדמת ומחפשים עסקים ראשונים. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום.
-אשמח לקפוץ ולהראות בכמה דקות. מתי מתאים?
+כאן [השם שלך] מפרקו. מאפייה היא המקום שאנשים חוזרים אליו הכי הרבה, ללחם של כל יום ולעוגה של שבת.
+פרקו היא אפליקציה אחת לכרטיסי מועדון של עסקים בשכונה. הלקוח סורק קוד בקופה וצובר חותמות לפי הכללים שלכם, למשל לחם עשירי עליכם, ורואה שם גם עסקים שכנים בעמק רפאים.
+אנחנו רוצים לחזק את העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כרגע אנחנו בגישה מוקדמת, וההצטרפות בחינם ובלי התחייבות.
+אשמח לקפוץ ולהראות את זה בכמה דקות. מתי מתאים?
 [השם שלך]</t>
         </is>
       </c>
@@ -2355,10 +2342,9 @@
       <c r="X17" s="9" t="inlineStr">
         <is>
           <t>היי ליאור ומתן,
-אני [השם שלך] מ-Perko. הדיינר שלכם הוא מקום שמשפחות ובני נוער חוזרים אליו, וזה בדיוק הקהל שכרטיס חותמות עובד אצלו הכי טוב.
-Perko הוא כרטיס נאמנות דיגיטלי משותף לעסקים בשכונה: הלקוח סורק קוד בקופה וצובר חותמות לפי ההטבה שאתם קובעים, למשל מילקשייק חינם בביקור השישי. באותה אפליקציה הוא רואה גם עסקים נוספים בעמק רפאים.
-פרקו נולדה כדי לשמור על העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כל ניקוב בכרטיס הוא עוד סיבה לחזור לעסק המקומי ולחזק את הקהילה שסביבו.
-אנחנו בגישה מוקדמת ומחפשים עסקים ראשונים. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום, ואם זה יעבוד אפשר יהיה להרחיב גם למקומות הנוספים שלכם.
+כאן [השם שלך] מפרקו. הדיינר שלכם הוא מקום שמשפחות ובני נוער חוזרים אליו, ושם כרטיס חותמות עובד הכי טוב.
+פרקו היא אפליקציה אחת לכרטיסי מועדון של עסקים בשכונה. הלקוח סורק קוד בקופה וצובר חותמות לפי הכללים שלכם, למשל מילקשייק חינם בביקור השישי.
+אנחנו רוצים לחזק את העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כרגע אנחנו בגישה מוקדמת, וההצטרפות בחינם ובלי התחייבות.
 אשמח לשיחה קצרה. מתי נוח?
 [השם שלך]</t>
         </is>
@@ -2473,11 +2459,10 @@
       <c r="X18" s="5" t="inlineStr">
         <is>
           <t>שלום אלישבע,
-אני [השם שלך] מ-Perko. קראתי עלייך ועל קומקום, ואהבתי את הבית הקטן והקהילתי שבנית בבקעה.
-אנחנו מפתחים כרטיס נאמנות דיגיטלי משותף לעסקים בשכונה: הלקוח סורק קוד בקופה וצובר חותמות לפי מה שתבחרי, למשל קנקן תה או סקונס במתנה, וגם קניות של תה עלים לבית נספרות. באותה אפליקציה הוא רואה גם עסקים שכנים בדרך בית לחם.
-פרקו נולדה כדי לשמור על העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כל ניקוב בכרטיס הוא עוד סיבה לחזור לעסק המקומי ולחזק את הקהילה שסביבו.
-אנחנו בגישה מוקדמת ומחפשים עסקים ראשונים. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום.
-אשמח לבוא לתה ולהראות בכמה דקות. מתי נוח לך?
+כאן [השם שלך] מפרקו. קראנו על קומקום ואהבנו את הבית הקטן והקהילתי שבנית בבקעה.
+פרקו היא אפליקציה אחת לכרטיסי מועדון של עסקים בשכונה. הלקוח סורק קוד בקופה וצובר חותמות לפי מה שתבחרי, למשל קנקן תה או סקונס במתנה, וגם קנייה של תה לבית יכולה להיספר.
+אנחנו רוצים לחזק את העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כרגע אנחנו בגישה מוקדמת, וההצטרפות בחינם ובלי התחייבות.
+אשמח לבוא לתה ולהראות את זה בכמה דקות. מתי נוח לך?
 [השם שלך]</t>
         </is>
       </c>
@@ -2575,11 +2560,10 @@
       <c r="X19" s="9" t="inlineStr">
         <is>
           <t>שלום לצוות פוקצ'ה במושבה,
-אני [השם שלך] מ-Perko. שוק הפוקצ'ות שלכם בשישי הוא בדיוק הרגל שבועי שכדאי לתגמל.
-אנחנו בונים כרטיס נאמנות דיגיטלי משותף לעסקים בעמק רפאים: הלקוח סורק קוד בקופה וצובר חותמות לפי ההטבה שאתם קובעים, למשל פוקצ'ה עלינו בשישי העשירי. באותה אפליקציה הוא רואה גם עסקים שכנים ברחוב.
-פרקו נולדה כדי לשמור על העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כל ניקוב בכרטיס הוא עוד סיבה לחזור לעסק המקומי ולחזק את הקהילה שסביבו.
-אנחנו בגישה מוקדמת ומחפשים עסקים ראשונים. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום.
-אשמח לדבר עם מי שמנהל את הסניף. מתי נוח?
+כאן [השם שלך] מפרקו. שוק הפוקצ'ות שלכם בשישי הוא בדיוק הרגל שבועי ששווה לתגמל.
+פרקו היא אפליקציה אחת לכרטיסי מועדון של עסקים בשכונה. הלקוח סורק קוד בקופה וצובר חותמות לפי הכללים שלכם, למשל פוקצ'ה עליכם בשישי העשירי.
+אנחנו רוצים לחזק את העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כרגע אנחנו בגישה מוקדמת, וההצטרפות בחינם ובלי התחייבות.
+אשמח לדבר עם מי שמנהל את המקום. מתי נוח?
 תודה,
 [השם שלך]</t>
         </is>
@@ -2678,10 +2662,9 @@
       <c r="X20" s="5" t="inlineStr">
         <is>
           <t>שלום לצוות פומפידו,
-אני [השם שלך] מ-Perko. אנחנו בונים כרטיס נאמנות דיגיטלי משותף לעסקים בעמק רפאים: הלקוח סורק קוד בקופה וצובר נקודות לפי ההטבה שאתם קובעים, למשל קינוח עלינו בביקור הרביעי.
-היתרון בשבילכם הוא החיבור לעסקים השכנים: לקוחות שמכירים את הרחוב מבתי הקפה ביום יכולים לגלות אתכם בערב דרך אותה אפליקציה.
-פרקו נולדה כדי לשמור על העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כל ניקוב בכרטיס הוא עוד סיבה לחזור לעסק המקומי ולחזק את הקהילה שסביבו.
-אנחנו בגישה מוקדמת ומחפשים עסקים ראשונים. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום.
+כאן [השם שלך] מפרקו. אנחנו בונים אפליקציה אחת לכרטיסי מועדון של עסקים בעמק רפאים, וחשבנו עליכם בגלל החיבור לשכנים ברחוב.
+לקוחות שמכירים את הרחוב מבתי הקפה ביום יכולים לגלות אתכם בערב דרך אותה אפליקציה. הם סורקים קוד בקופה וצוברים נקודות לפי ההטבה שאתם קובעים, למשל קינוח עליכם בביקור הרביעי.
+אנחנו רוצים לחזק את העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כרגע אנחנו בגישה מוקדמת, וההצטרפות בחינם ובלי התחייבות.
 אשמח לדבר עם מי שמנהל את המקום. מתי אפשר לתפוס אתכם?
 תודה,
 [השם שלך]</t>
@@ -2781,10 +2764,9 @@
       <c r="X21" s="9" t="inlineStr">
         <is>
           <t>שלום לצוות רנדבו,
-אני [השם שלך] מ-Perko. פיצה ופסטה הן הזמנות שמשפחות חוזרות אליהן שוב ושוב, וזה בדיוק המקום שבו כרטיס חותמות עובד.
-Perko הוא כרטיס נאמנות דיגיטלי משותף לעסקים בדרך בית לחם: הלקוח סורק קוד בקופה וצובר חותמות לפי ההטבה שאתם קובעים, ובאותה אפליקציה רואה גם עסקים נוספים ברחוב.
-פרקו נולדה כדי לשמור על העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כל ניקוב בכרטיס הוא עוד סיבה לחזור לעסק המקומי ולחזק את הקהילה שסביבו.
-אנחנו בגישה מוקדמת ומחפשים עסקים ראשונים. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום.
+כאן [השם שלך] מפרקו. פיצה ופסטה הן הזמנות שמשפחות חוזרות אליהן שוב ושוב, ושם כרטיס חותמות עובד הכי טוב.
+פרקו היא אפליקציה אחת לכרטיסי מועדון של עסקים בשכונה. הלקוח סורק קוד בקופה וצובר חותמות לפי הכללים שלכם, ורואה שם גם עסקים נוספים בדרך בית לחם.
+אנחנו רוצים לחזק את העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כרגע אנחנו בגישה מוקדמת, וההצטרפות בחינם ובלי התחייבות.
 אשמח לשיחה קצרה עם מי שמנהל את המקום. מתי נוח?
 [השם שלך]</t>
         </is>
@@ -2891,10 +2873,9 @@
       <c r="X22" s="5" t="inlineStr">
         <is>
           <t>שלום ברברה,
-אני [השם שלך] מ-Perko. אנחנו בונים כרטיס נאמנות דיגיטלי משותף לעסקים בעמק רפאים: הלקוח סורק קוד בקופה, צובר הטבות לפי הכללים של כל עסק, ורואה באותה אפליקציה את כל העסקים המשתתפים ברחוב.
-בשביל חנות מתנות היתרון העיקרי הוא החשיפה: לקוחות קבועים של בתי הקפה והמאפיות ברחוב יכולים לגלות אתכם, במיוחד לפני החגים. ההטבה יכולה להיות משהו קטן, כמו עטיפת מתנה או הנחה לקנייה הבאה.
-פרקו נולדה כדי לשמור על העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כל ניקוב בכרטיס הוא עוד סיבה לחזור לעסק המקומי ולחזק את הקהילה שסביבו.
-אנחנו בגישה מוקדמת. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום.
+כאן [השם שלך] מפרקו. אנחנו בונים אפליקציה אחת לכרטיסי מועדון של עסקים בעמק רפאים, וחשבנו על החנות שלך.
+בשביל חנות מתנות היתרון הוא החשיפה: לקוחות קבועים של בתי הקפה והמאפיות ברחוב יכולים לגלות אותך, במיוחד לפני החגים. ההטבה יכולה להיות קטנה, כמו עטיפת מתנה או הנחה לקנייה הבאה.
+אנחנו רוצים לחזק את העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כרגע אנחנו בגישה מוקדמת, וההצטרפות בחינם ובלי התחייבות.
 אשמח לשמוע אם זה מעניין אותך.
 תודה,
 [השם שלך]</t>
@@ -3018,10 +2999,9 @@
       <c r="X23" s="9" t="inlineStr">
         <is>
           <t>שלום דליה ואייל,
-אני [השם שלך] מ-Perko. סתיו תכשיטים הוא מהעסקים הוותיקים והמיוחדים בעמק רפאים, וזה בדיוק סוג המקום שאנחנו רוצים שאנשים מהשכונה יגלו.
-אנחנו בונים כרטיס נאמנות דיגיטלי משותף לעסקים ברחוב. אצלכם זה לא יהיה כרטיס חותמות רגיל: אפשר להגדיר הטבה שמתאימה לתכשיטים, כמו ניקוי, תיקון או חריטה במתנה, ולהגיע ללקוחות של בתי הקפה והחנויות השכנות באותה אפליקציה.
-פרקו נולדה כדי לשמור על העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כל ניקוב בכרטיס הוא עוד סיבה לחזור לעסק המקומי ולחזק את הקהילה שסביבו.
-אנחנו בגישה מוקדמת. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום.
+כאן [השם שלך] מפרקו. סתיו תכשיטים הוא מהעסקים הוותיקים והמיוחדים בעמק רפאים, בדיוק מהמקומות שאנחנו רוצים שאנשים מהשכונה יגלו.
+פרקו היא אפליקציה אחת לכרטיסי מועדון של עסקים ברחוב. אצלכם זה לא חייב להיות כרטיס חותמות רגיל: אפשר להגדיר הטבה שמתאימה לתכשיטים, כמו ניקוי, תיקון או חריטה במתנה.
+אנחנו רוצים לחזק את העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כרגע אנחנו בגישה מוקדמת, וההצטרפות בחינם ובלי התחייבות.
 אשמח לשמוע אם זה מעניין אתכם, ולקפוץ לשיחה קצרה.
 תודה,
 [השם שלך]</t>

</xml_diff>

<commit_message>
Research: WhatsApp and email versions of every outreach message, with send tracking
Each business gets a short WhatsApp note and a fuller email with a subject.
The page adds sent/replied checkboxes with dates, notes, progress, status
filter and CSV export (stored in the browser).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VZAuLHaESUH9foWg6jPqbt
</commit_message>
<xml_diff>
--- a/research/Perko_Local_Business_Prospects_Jerusalem.xlsx
+++ b/research/Perko_Local_Business_Prospects_Jerusalem.xlsx
@@ -887,11 +887,17 @@
       <c r="X4" s="5" t="inlineStr">
         <is>
           <t>היי מיכאל ודניאל,
-כאן [השם שלך] מפרקו. בירמה היא בדיוק סוג המקום שאנחנו בונים בשבילו: קלייה קטנה ודלפק עם לקוחות קבועים שעוצרים בדרך לעבודה.
-פרקו מחליפה את כרטיס הנייר באפליקציה אחת לכל העסקים בשכונה. הלקוח סורק קוד בקופה, צובר חותמות לפי הכללים שלכם, ורואה שם גם עסקים נוספים ברחוב.
-אנחנו רוצים לחזק את העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כרגע אנחנו בגישה מוקדמת, וההצטרפות בחינם ובלי התחייבות.
-יש לכם רבע שעה השבוע? אשמח להגיע לדלפק.
-[השם שלך]</t>
+כאן [השם שלך] מפרקו. ראינו מה בניתם בבירמה מאז 2021: קלייה קטנה, דלפק טייק-אוויי ולקוחות קבועים שעוצרים בדרך לעבודה. זה בדיוק העסק שכרטיס חותמות נועד בשבילו.
+פרקו היא אפליקציה אחת לכרטיסי מועדון של עסקים שכונתיים. במקום כרטיס נייר, הלקוח סורק קוד בקופה, צובר חותמות לפי הכללים שאתם קובעים, ורואה באותה אפליקציה גם עסקים שכנים בעמק רפאים.
+מה זה יכול לתת לבירמה:
+- כרטיס חותמות בלי נייר ובלי הדפסות: קפה עשירי עליכם, או כל כלל אחר שתחליטו.
+- לקוח הבוקר רואה בטלפון שחסרות לו שתי חותמות, וזו עוד סיבה לעצור דווקא אצלכם.
+- מקום ראשון ברשת של עסקים שכונתיים ברחוב, כמותג צעיר שמשפיע על איך המוצר ייראה.
+אנחנו בשלב גישה מוקדמת ומחפשים כמה עסקים ראשונים בעמק רפאים שיעזרו לנו לבנות את זה נכון. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום, ונעזור אתכם בהקמה. המטרה שלנו פשוטה: לחזק את העסקים הקטנים והמשפחתיים שעושים את השכונה לבית.
+יש לכם רבע שעה השבוע? אשמח להגיע לדלפק ולהראות.
+תודה,
+[השם שלך]
+פרקו · getperko.com</t>
         </is>
       </c>
     </row>
@@ -1004,12 +1010,17 @@
       <c r="X5" s="9" t="inlineStr">
         <is>
           <t>שלום לצוות קאלו,
-כאן [השם שלך] מפרקו. קאלו הוא כבר שנים חלק מהשגרה של בקעה, גם בבית הקפה וגם במעדנייה.
-פרקו היא אפליקציה אחת לכרטיסי מועדון של עסקים בשכונה. הלקוח סורק קוד בקופה וצובר חותמות לפי הכללים שלכם, למשל ארוחת בוקר עשירית עליכם. באותה אפליקציה הלקוח רואה גם עסקים נוספים בדרך בית לחם.
-אנחנו רוצים לחזק את העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כרגע אנחנו בגישה מוקדמת, וההצטרפות בחינם ובלי התחייבות.
-אשמח לדבר עם מי שאחראי אצלכם על הלקוחות. למי כדאי לפנות?
+כאן [השם שלך] מפרקו. קאלו הוא כבר יותר מעשרים וחמש שנה חלק מהשגרה של בקעה, עם קהל מקומי גדול שמגיע גם לארוחת בוקר וגם לקניות במעדנייה.
+פרקו היא אפליקציה אחת לכרטיסי מועדון של עסקים שכונתיים. במקום כרטיס נייר, הלקוח סורק קוד בקופה, צובר חותמות או נקודות לפי ההטבה שאתם מגדירים, ורואה באותה אפליקציה גם עסקים שכנים בדרך בית לחם.
+מה זה יכול לתת לקאלו:
+- הטבה אחת פשוטה שמתאימה לשני סוגי הקנייה, למשל נקודות על כל קנייה ומנה מוכנה או ארוחת בוקר במתנה.
+- קשר דיגיטלי עם הקבועים, בלי לבנות אפליקציה משלכם.
+- קאלו יכול להיות עוגן של הרשת בדרך בית לחם, יחד עם השכנים ברחוב.
+אנחנו בשלב גישה מוקדמת ומחפשים כמה עסקים ראשונים בדרך בית לחם שיעזרו לנו לבנות את זה נכון. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום, ונעזור אתכם בהקמה. המטרה שלנו פשוטה: לחזק את העסקים הקטנים והמשפחתיים שעושים את השכונה לבית.
+אשמח לדבר עם מי שאחראי אצלכם על הלקוחות, או לקפוץ ולהראות. למי כדאי לפנות?
 תודה,
-[השם שלך]</t>
+[השם שלך]
+פרקו · getperko.com</t>
         </is>
       </c>
     </row>
@@ -1130,12 +1141,17 @@
       <c r="X6" s="5" t="inlineStr">
         <is>
           <t>שלום לאה ואבי,
-כאן [השם שלך] מפרקו. טחנת הקפה היא מהמקומות שאנשים בעמק רפאים חוזרים אליהם כל בוקר, וגם לשקית הפולים כל כמה שבועות.
-פרקו היא אפליקציה אחת לכרטיסי מועדון של עסקים בשכונה. הלקוח סורק קוד בקופה וצובר חותמות לפי הכללים שלכם, למשל קפה עשירי עליכם או הנחה על שקית פולים.
-אנחנו רוצים לחזק את העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כרגע אנחנו בגישה מוקדמת, וההצטרפות בחינם ובלי התחייבות.
-אשמח לקפוץ לקפה ולהראות לכם את זה בעשר דקות. מתי נוח?
+כאן [השם שלך] מפרקו. אתם קולים קפה במושבה הגרמנית כבר שלושים שנה, ויש לכם בדיוק את מה שכרטיס מועדון נבנה בשבילו: לקוחות שחוזרים כל בוקר, וגם קונים שוב את הפולים כל כמה שבועות.
+פרקו היא אפליקציה אחת לכרטיסי מועדון של עסקים שכונתיים. במקום כרטיס נייר, הלקוח סורק קוד בקופה, צובר חותמות לפי הכללים שאתם קובעים, ורואה באותה אפליקציה גם עסקים שכנים בעמק רפאים.
+מה זה יכול לתת לטחנת הקפה:
+- תגמול לשני סוגי החזרה: קפה עשירי עליכם, ובנוסף הטבה על כל שקית פולים רביעית.
+- סוף לכרטיסי נייר שנשכחים בארנק: הלקוח רואה בטלפון כמה חסר לו להטבה.
+- חשיפה ללקוחות של עסקים שכנים ברחוב שמשתמשים באותה אפליקציה.
+אנחנו בשלב גישה מוקדמת ומחפשים כמה עסקים ראשונים בעמק רפאים שיעזרו לנו לבנות את זה נכון. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום, ונעזור אתכם בהקמה. המטרה שלנו פשוטה: לחזק את העסקים הקטנים והמשפחתיים שעושים את השכונה לבית.
+אשמח לקפוץ לקפה ולהראות לכם את זה בעשר דקות. מתי נוח לכם?
 תודה,
-[השם שלך]</t>
+[השם שלך]
+פרקו · getperko.com</t>
         </is>
       </c>
     </row>
@@ -1248,11 +1264,17 @@
       <c r="X7" s="9" t="inlineStr">
         <is>
           <t>היי מיטל ואלפונסו,
-כאן [השם שלך] מפרקו. אהבנו את מה שבניתם בקאסה לביא: קלייה משלכם, מאפים בריאים וקהל שחוזר כמה פעמים בשבוע.
-פרקו היא אפליקציה אחת לכרטיסי מועדון של עסקים בשכונה. הלקוח סורק קוד בקופה וצובר חותמות לפי הכללים שלכם, ורואה שם גם עסקים שכנים בדרך בית לחם.
-אנחנו רוצים לחזק את העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כרגע אנחנו בגישה מוקדמת, וההצטרפות בחינם ובלי התחייבות.
+כאן [השם שלך] מפרקו. אהבנו את מה שבניתם בקאסה לביא: קלייה משלכם, מאפים בלי סוכר לבן ובלי קמח לבן, וקהל שחוזר כמה פעמים בשבוע.
+פרקו היא אפליקציה אחת לכרטיסי מועדון של עסקים שכונתיים. במקום כרטיס נייר, הלקוח סורק קוד בקופה, צובר חותמות לפי הכללים שאתם קובעים, ורואה באותה אפליקציה גם עסקים שכנים בדרך בית לחם.
+מה זה יכול לתת לקאסה לביא:
+- תגמול לקהל הקבוע, בכללים שאתם בוחרים: קפה, מאפה, או שילוב.
+- חשיפה ללקוחות של עסקים שכנים שמחפשים בדיוק מקום כמו שלכם.
+- השפעה על המוצר מההתחלה, כעסק צעיר שמוביל את הפיילוט.
+אנחנו בשלב גישה מוקדמת ומחפשים כמה עסקים ראשונים בדרך בית לחם שיעזרו לנו לבנות את זה נכון. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום, ונעזור אתכם בהקמה. המטרה שלנו פשוטה: לחזק את העסקים הקטנים והמשפחתיים שעושים את השכונה לבית.
 אשמח לקפוץ לקפה ולהראות את זה בכמה דקות. מתי נוח לכם?
-[השם שלך]</t>
+תודה,
+[השם שלך]
+פרקו · getperko.com</t>
         </is>
       </c>
     </row>
@@ -1353,11 +1375,17 @@
       <c r="X8" s="5" t="inlineStr">
         <is>
           <t>שלום לצוות פרחי העמק,
-כאן [השם שלך] מפרקו. הרבה משפחות בשכונה קונות פרחים לשבת כל שבוע, וזה בדיוק הלקוח הקבוע שאנחנו בונים בשבילו.
-פרקו היא אפליקציה אחת לכרטיסי מועדון של עסקים בשכונה. הלקוח סורק קוד בקופה וצובר חותמות לפי הכללים שלכם, למשל זר תשיעי במתנה. באותה אפליקציה הוא רואה גם את בתי הקפה והחנויות השכנות בעמק רפאים.
-אנחנו רוצים לחזק את העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כרגע אנחנו בגישה מוקדמת, וההצטרפות בחינם ובלי התחייבות.
-אשמח לעשר דקות שיחה או לקפוץ לחנות. מתי מתאים?
-[השם שלך]</t>
+כאן [השם שלך] מפרקו. הרבה משפחות במושבה קונות פרחים לשבת כל שבוע, וזה בדיוק הלקוח הקבוע שכרטיס מועדון נבנה בשבילו.
+פרקו היא אפליקציה אחת לכרטיסי מועדון של עסקים שכונתיים. במקום כרטיס נייר, הלקוח סורק קוד בקופה, צובר חותמות לפי הכללים שאתם קובעים, ורואה באותה אפליקציה גם עסקים שכנים בעמק רפאים.
+מה זה יכול לתת לפרחי העמק:
+- הטבה שמתאימה להרגל של שישי, למשל שמונה זרים והתשיעי במתנה.
+- לקוחות של בתי הקפה ברחוב יכולים לגלות אתכם באותה אפליקציה, כעצירה שנייה בדרך הביתה.
+- בלי כרטיסים מודפסים ובלי מערכת חדשה לתפעל בחנות.
+אנחנו בשלב גישה מוקדמת ומחפשים כמה עסקים ראשונים בעמק רפאים שיעזרו לנו לבנות את זה נכון. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום, ונעזור אתכם בהקמה. המטרה שלנו פשוטה: לחזק את העסקים הקטנים והמשפחתיים שעושים את השכונה לבית.
+אשמח לעשר דקות שיחה או לקפוץ לחנות. מתי מתאים לכם?
+תודה,
+[השם שלך]
+פרקו · getperko.com</t>
         </is>
       </c>
     </row>
@@ -1458,11 +1486,17 @@
       <c r="X9" s="9" t="inlineStr">
         <is>
           <t>שלום לצוות של המקום של איציק,
-כאן [השם שלך] מפרקו. אתם מהמקומות שהשכונה חוזרת אליהם כל יום, עוד מימי הקיוסק.
-פרקו היא כרטיס מועדון דיגיטלי אחד לעסקים בדרך בית לחם, בלי כרטיס נייר ובלי אפליקציה נפרדת. הלקוח סורק קוד בקופה וצובר חותמות לפי מה שתחליטו, למשל קפה עשירי חינם.
-אנחנו רוצים לחזק את העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כרגע אנחנו בגישה מוקדמת, וההצטרפות בחינם ובלי התחייבות.
-אפשר לקפוץ אליכם לכמה דקות בשעה שקטה? מתי הכי נוח?
-[השם שלך]</t>
+כאן [השם שלך] מפרקו. אתם מהמקומות שהשכונה חוזרת אליהם כל יום, עוד מימי הקיוסק, ובלי שום אפליקציה או אתר משלכם.
+פרקו היא אפליקציה אחת לכרטיסי מועדון של עסקים שכונתיים. במקום כרטיס נייר, הלקוח סורק קוד בקופה, צובר חותמות לפי הכללים שאתם קובעים, ורואה באותה אפליקציה גם עסקים שכנים בדרך בית לחם.
+מה זה יכול לתת להמקום של איציק:
+- כרטיס קפה דיגיטלי מוכן, בלי לפתח כלום ובלי לנהל אתר: מדפיסים קוד לקופה וזהו.
+- הקבועים שלכם רואים בטלפון כמה חסר להם, ולא מאבדים כרטיסי נייר.
+- אתם שתי דלתות מקאלו ומציגה, וביחד אפשר לבנות רחוב שבו כל עצירה נספרת.
+אנחנו בשלב גישה מוקדמת ומחפשים כמה עסקים ראשונים בדרך בית לחם שיעזרו לנו לבנות את זה נכון. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום, ונעזור אתכם בהקמה. המטרה שלנו פשוטה: לחזק את העסקים הקטנים והמשפחתיים שעושים את השכונה לבית.
+אפשר לקפוץ אליכם לכמה דקות בשעה שקטה ולהראות? מה הזמן הכי נוח?
+תודה,
+[השם שלך]
+פרקו · getperko.com</t>
         </is>
       </c>
     </row>
@@ -1567,12 +1601,17 @@
       <c r="X10" s="5" t="inlineStr">
         <is>
           <t>שלום לצוות ציגה,
-כאן [השם שלך] מפרקו. גלידה היא בדיוק הפינוק שמשפחות מהשכונה חוזרות אליו שוב ושוב.
-פרקו היא אפליקציה אחת לכרטיסי מועדון של עסקים בשכונה. הלקוח סורק קוד בקופה וצובר חותמות לפי הכללים שלכם, למשל ״כל כדור שמיני עלינו״.
-אנחנו רוצים לחזק את העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כרגע אנחנו בגישה מוקדמת, וההצטרפות בחינם ובלי התחייבות.
-אשמח לשיחה קצרה או לקפוץ אליכם. מתי נוח?
+כאן [השם שלך] מפרקו. ג'לאטו בעבודת יד הוא בדיוק הפינוק שמשפחות מהשכונה חוזרות אליו שוב ושוב, וזה המקום שבו כרטיס חותמות הכי קל להבנה.
+פרקו היא אפליקציה אחת לכרטיסי מועדון של עסקים שכונתיים. במקום כרטיס נייר, הלקוח סורק קוד בקופה, צובר חותמות לפי הכללים שאתם קובעים, ורואה באותה אפליקציה גם עסקים שכנים בדרך בית לחם.
+מה זה יכול לתת לציגה:
+- הטבה שילדים ומבוגרים מבינים מיד, למשל ״כל כדור שמיני עלינו״.
+- המשפחה רואה בטלפון שחסר להם עוד ביקור אחד, ויש סיבה לבוא שוב בשבוע הבא.
+- אתם באותו בניין עם קאלו, כך שלקוח יכול לצבור אצל שניכם באותה יציאה.
+אנחנו בשלב גישה מוקדמת ומחפשים כמה עסקים ראשונים בדרך בית לחם שיעזרו לנו לבנות את זה נכון. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום, ונעזור אתכם בהקמה. המטרה שלנו פשוטה: לחזק את העסקים הקטנים והמשפחתיים שעושים את השכונה לבית.
+אשמח לשיחה קצרה או לקפוץ אליכם. מתי נוח לכם?
 תודה,
-[השם שלך]</t>
+[השם שלך]
+פרקו · getperko.com</t>
         </is>
       </c>
     </row>
@@ -1673,11 +1712,17 @@
       <c r="X11" s="9" t="inlineStr">
         <is>
           <t>שלום לצוות ברזאולה,
-כאן [השם שלך] מפרקו. יש לכם קהל נאמן אמיתי, שמגיע גם לקניות הביתה וגם לערב בבר.
-פרקו היא אפליקציה אחת לכרטיסי מועדון של עסקים בשכונה. הלקוח סורק קוד בקופה וצובר חותמות לפי הכללים שלכם, ורואה שם גם עסקים שכנים בדרך בית לחם.
-אנחנו רוצים לחזק את העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כרגע אנחנו בגישה מוקדמת, וההצטרפות בחינם ובלי התחייבות.
+כאן [השם שלך] מפרקו. יש לכם קהל נאמן אמיתי, שמגיע גם לנקניקים לבית וגם לערב של טאפאס בבר.
+פרקו היא אפליקציה אחת לכרטיסי מועדון של עסקים שכונתיים. במקום כרטיס נייר, הלקוח סורק קוד בקופה, צובר חותמות לפי הכללים שאתם קובעים, ורואה באותה אפליקציה גם עסקים שכנים בדרך בית לחם.
+מה זה יכול לתת לברזאולה:
+- כרטיס אחד שסופר גם קנייה בדלפק וגם ערב בבר.
+- הטבה שמחזירה את מי שבא פעם בחודש להיות קבוע, למשל מנת טאפאס במתנה.
+- חשיפה ללקוחות של בתי הקפה והמעדניות ברחוב.
+אנחנו בשלב גישה מוקדמת ומחפשים כמה עסקים ראשונים בדרך בית לחם שיעזרו לנו לבנות את זה נכון. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום, ונעזור אתכם בהקמה. המטרה שלנו פשוטה: לחזק את העסקים הקטנים והמשפחתיים שעושים את השכונה לבית.
 אשמח לקפוץ אליכם לכמה דקות. מתי הכי שקט אצלכם?
-[השם שלך]</t>
+תודה,
+[השם שלך]
+פרקו · getperko.com</t>
         </is>
       </c>
     </row>
@@ -1786,12 +1831,17 @@
       <c r="X12" s="5" t="inlineStr">
         <is>
           <t>שלום לצוות הפרחים של ארז,
-כאן [השם שלך] מפרקו. יש לכם גם קונים שנכנסים לפני שבת וגם לקוחות משלוחים שחוזרים, וזה בדיוק הקהל שאנחנו בונים בשבילו.
-פרקו היא אפליקציה אחת לכרטיסי מועדון של עסקים בשכונה. הלקוח סורק קוד בקופה וצובר חותמות לפי הכללים שלכם, ורואה שם גם עסקים נוספים בעמק רפאים.
-אנחנו רוצים לחזק את העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כרגע אנחנו בגישה מוקדמת, וההצטרפות בחינם ובלי התחייבות.
+כאן [השם שלך] מפרקו. יש לכם גם קונים שנכנסים לחנות לפני שבת וגם לקוחות משלוחים שחוזרים שוב ושוב, וזה בדיוק הקהל שכרטיס מועדון נבנה בשבילו.
+פרקו היא אפליקציה אחת לכרטיסי מועדון של עסקים שכונתיים. במקום כרטיס נייר, הלקוח סורק קוד בקופה, צובר חותמות לפי הכללים שאתם קובעים, ורואה באותה אפליקציה גם עסקים שכנים בעמק רפאים.
+מה זה יכול לתת להפרחים של ארז:
+- הטבה ללקוחות שחוזרים, למשל זר במתנה אחרי כמה קניות.
+- הלקוח רואה בטלפון כמה חסר לו, ולא צריך לשמור כרטיס.
+- חשיפה ללקוחות של בתי הקפה והמאפיות בעמק רפאים.
+אנחנו בשלב גישה מוקדמת ומחפשים כמה עסקים ראשונים בעמק רפאים שיעזרו לנו לבנות את זה נכון. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום, ונעזור אתכם בהקמה. המטרה שלנו פשוטה: לחזק את העסקים הקטנים והמשפחתיים שעושים את השכונה לבית.
 אשמח לעשר דקות שיחה. מתי נוח לכם?
 תודה,
-[השם שלך]</t>
+[השם שלך]
+פרקו · getperko.com</t>
         </is>
       </c>
     </row>
@@ -1896,12 +1946,17 @@
       <c r="X13" s="9" t="inlineStr">
         <is>
           <t>שלום לצוות פלורה,
-כאן [השם שלך] מפרקו. פרחים לשבת ולחגים הם בדיוק קנייה שחוזרת על עצמה, ושווה לתגמל עליה.
-פרקו היא אפליקציה אחת לכרטיסי מועדון של עסקים בשכונה. הלקוח סורק קוד בקופה וצובר חותמות לפי הכללים שלכם, למשל זר תשיעי במתנה. באותה אפליקציה הוא רואה גם בתי קפה ועסקים שכנים בדרך בית לחם.
-אנחנו רוצים לחזק את העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כרגע אנחנו בגישה מוקדמת, וההצטרפות בחינם ובלי התחייבות.
+כאן [השם שלך] מפרקו. פרחים לשבת, ועוד שיאים בחגים, הם בדיוק קנייה שחוזרת על עצמה ושווה לתגמל עליה.
+פרקו היא אפליקציה אחת לכרטיסי מועדון של עסקים שכונתיים. במקום כרטיס נייר, הלקוח סורק קוד בקופה, צובר חותמות לפי הכללים שאתם קובעים, ורואה באותה אפליקציה גם עסקים שכנים בדרך בית לחם.
+מה זה יכול לתת לפלורה:
+- הטבה שמתאימה לשישי, למשל זר תשיעי במתנה, שנספרת גם באיסוף מהחנות.
+- אתם כמה דלתות מקאלו ומציגה, אז לקוח יכול לצבור אצל כמה עסקים באותו סיבוב.
+- בלי כרטיסים מודפסים ובלי מערכת חדשה לתפעל.
+אנחנו בשלב גישה מוקדמת ומחפשים כמה עסקים ראשונים בדרך בית לחם שיעזרו לנו לבנות את זה נכון. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום, ונעזור אתכם בהקמה. המטרה שלנו פשוטה: לחזק את העסקים הקטנים והמשפחתיים שעושים את השכונה לבית.
 אשמח לשיחה קצרה או לקפוץ לחנות. מתי נוח לכם?
 תודה,
-[השם שלך]</t>
+[השם שלך]
+פרקו · getperko.com</t>
         </is>
       </c>
     </row>
@@ -2018,12 +2073,17 @@
       <c r="X14" s="5" t="inlineStr">
         <is>
           <t>שלום עדי ושרה,
-כאן [השם שלך] מפרקו. גראנד קפה הוא מהמקומות שמגדירים את בקעה, עם קהל בראנץ' נאמן.
-פרקו היא אפליקציה אחת לכרטיסי מועדון של עסקים בשכונה. הלקוח סורק קוד בקופה וצובר חותמות לפי הכללים שלכם, למשל מאפה עליכם בביקור באמצע השבוע.
-אנחנו רוצים לחזק את העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כרגע אנחנו בגישה מוקדמת, וההצטרפות בחינם ובלי התחייבות.
-אשמח לפגישה קצרה בזמן שנוח לכם.
+כאן [השם שלך] מפרקו. גראנד קפה הוא מהמקומות שמגדירים את בקעה כבר מ-2011, עם קהל בראנץ' ומאפים נאמן.
+פרקו היא אפליקציה אחת לכרטיסי מועדון של עסקים שכונתיים. במקום כרטיס נייר, הלקוח סורק קוד בקופה, צובר חותמות לפי הכללים שאתם קובעים, ורואה באותה אפליקציה גם עסקים שכנים בדרך בית לחם.
+מה זה יכול לתת לגראנד קפה:
+- הטבה שמזיזה ביקורים, למשל מאפה עליכם למי שמגיע גם באמצע השבוע.
+- קשר דיגיטלי עם הקבועים של סוף השבוע, בלי אפליקציה נפרדת.
+- מקום מוכר כמו שלכם נותן לרשת השכונתית אמינות, ומקבל ממנה לקוחות של העסקים השכנים.
+אנחנו בשלב גישה מוקדמת ומחפשים כמה עסקים ראשונים בדרך בית לחם שיעזרו לנו לבנות את זה נכון. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום, ונעזור אתכם בהקמה. המטרה שלנו פשוטה: לחזק את העסקים הקטנים והמשפחתיים שעושים את השכונה לבית.
+אשמח לפגישה קצרה בזמן שנוח לכם. מתי מתאים?
 תודה,
-[השם שלך]</t>
+[השם שלך]
+פרקו · getperko.com</t>
         </is>
       </c>
     </row>
@@ -2128,11 +2188,17 @@
       <c r="X15" s="9" t="inlineStr">
         <is>
           <t>שלום לצוות לה שרולה,
-כאן [השם שלך] מפרקו. הרבה משפחות בשכונה קונות אצלכם לשבת כל שבוע, וזה בדיוק הלקוח הקבוע שאנחנו בונים בשבילו.
-פרקו היא אפליקציה אחת לכרטיסי מועדון של עסקים בשכונה. הלקוח סורק קוד בקופה וצובר נקודות לפי הכללים שלכם, ורואה שם גם עסקים נוספים בדרך בית לחם.
-אנחנו רוצים לחזק את העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כרגע אנחנו בגישה מוקדמת, וההצטרפות בחינם ובלי התחייבות.
+כאן [השם שלך] מפרקו. הרבה משפחות בבקעה קונות אצלכם לשבת כל שבוע, וזה בדיוק הלקוח הקבוע שכרטיס מועדון נבנה בשבילו.
+פרקו היא אפליקציה אחת לכרטיסי מועדון של עסקים שכונתיים. במקום כרטיס נייר, הלקוח סורק קוד בקופה, צובר חותמות או נקודות לפי הכללים שאתם קובעים, ורואה באותה אפליקציה גם עסקים שכנים בדרך בית לחם.
+מה זה יכול לתת ללה שרולה:
+- נקודות לפי גובה הקנייה, שמתאימות לסלים הגדולים של סוף השבוע.
+- הטבה שמחזקת את ההרגל השבועי, למשל מנה מוכנה או מאפה צרפתי במתנה.
+- אתם עסק שונה מבתי הקפה ברחוב, וזה בדיוק מה שהופך רשת שכונתית לשימושית.
+אנחנו בשלב גישה מוקדמת ומחפשים כמה עסקים ראשונים בדרך בית לחם שיעזרו לנו לבנות את זה נכון. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום, ונעזור אתכם בהקמה. המטרה שלנו פשוטה: לחזק את העסקים הקטנים והמשפחתיים שעושים את השכונה לבית.
 אשמח לשיחה קצרה עם מי שמנהל את החנות. מתי נוח?
-[השם שלך]</t>
+תודה,
+[השם שלך]
+פרקו · getperko.com</t>
         </is>
       </c>
     </row>
@@ -2229,11 +2295,17 @@
       <c r="X16" s="5" t="inlineStr">
         <is>
           <t>שלום לצוות לחם ועוד,
-כאן [השם שלך] מפרקו. מאפייה היא המקום שאנשים חוזרים אליו הכי הרבה, ללחם של כל יום ולעוגה של שבת.
-פרקו היא אפליקציה אחת לכרטיסי מועדון של עסקים בשכונה. הלקוח סורק קוד בקופה וצובר חותמות לפי הכללים שלכם, למשל לחם עשירי עליכם, ורואה שם גם עסקים שכנים בעמק רפאים.
-אנחנו רוצים לחזק את העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כרגע אנחנו בגישה מוקדמת, וההצטרפות בחינם ובלי התחייבות.
-אשמח לקפוץ ולהראות את זה בכמה דקות. מתי מתאים?
-[השם שלך]</t>
+כאן [השם שלך] מפרקו. מאפייה היא המקום שאנשים חוזרים אליו הכי הרבה, ללחם המחמצת של כל יום ולעוגת הגבינה של שבת.
+פרקו היא אפליקציה אחת לכרטיסי מועדון של עסקים שכונתיים. במקום כרטיס נייר, הלקוח סורק קוד בקופה, צובר חותמות לפי הכללים שאתם קובעים, ורואה באותה אפליקציה גם עסקים שכנים בעמק רפאים.
+מה זה יכול לתת ללחם ועוד:
+- כרטיס פשוט ללחם היומי, למשל לחם עשירי עליכם.
+- הטבה עשירה יותר לקניות הגדולות במעדנייה, לפי מה שתחליטו.
+- חשיפה ללקוחות של בתי הקפה וחנויות הפרחים ברחוב.
+אנחנו בשלב גישה מוקדמת ומחפשים כמה עסקים ראשונים בעמק רפאים שיעזרו לנו לבנות את זה נכון. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום, ונעזור אתכם בהקמה. המטרה שלנו פשוטה: לחזק את העסקים הקטנים והמשפחתיים שעושים את השכונה לבית.
+אשמח לקפוץ ולהראות את זה בכמה דקות. מתי מתאים לכם?
+תודה,
+[השם שלך]
+פרקו · getperko.com</t>
         </is>
       </c>
     </row>
@@ -2342,11 +2414,17 @@
       <c r="X17" s="9" t="inlineStr">
         <is>
           <t>היי ליאור ומתן,
-כאן [השם שלך] מפרקו. הדיינר שלכם הוא מקום שמשפחות ובני נוער חוזרים אליו, ושם כרטיס חותמות עובד הכי טוב.
-פרקו היא אפליקציה אחת לכרטיסי מועדון של עסקים בשכונה. הלקוח סורק קוד בקופה וצובר חותמות לפי הכללים שלכם, למשל מילקשייק חינם בביקור השישי.
-אנחנו רוצים לחזק את העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כרגע אנחנו בגישה מוקדמת, וההצטרפות בחינם ובלי התחייבות.
-אשמח לשיחה קצרה. מתי נוח?
-[השם שלך]</t>
+כאן [השם שלך] מפרקו. הדיינר שלכם הוא מקום שמשפחות ובני נוער חוזרים אליו, וזה בדיוק הקהל שכרטיס חותמות עובד אצלו הכי טוב.
+פרקו היא אפליקציה אחת לכרטיסי מועדון של עסקים שכונתיים. במקום כרטיס נייר, הלקוח סורק קוד בקופה, צובר חותמות לפי הכללים שאתם קובעים, ורואה באותה אפליקציה גם עסקים שכנים בעמק רפאים.
+מה זה יכול לתת לבוכמן'ס:
+- הטבה שקל להסביר לכל שולחן, למשל מילקשייק חינם בביקור השישי.
+- בני נוער שכבר חיים בטלפון מקבלים כרטיס שלא נאבד.
+- אם זה יעבוד אצלכם, אפשר יהיה לבחון את זה גם במקומות האחרים שלכם.
+אנחנו בשלב גישה מוקדמת ומחפשים כמה עסקים ראשונים בעמק רפאים שיעזרו לנו לבנות את זה נכון. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום, ונעזור אתכם בהקמה. המטרה שלנו פשוטה: לחזק את העסקים הקטנים והמשפחתיים שעושים את השכונה לבית.
+אשמח לשיחה קצרה. מתי נוח לכם?
+תודה,
+[השם שלך]
+פרקו · getperko.com</t>
         </is>
       </c>
     </row>
@@ -2459,11 +2537,17 @@
       <c r="X18" s="5" t="inlineStr">
         <is>
           <t>שלום אלישבע,
-כאן [השם שלך] מפרקו. קראנו על קומקום ואהבנו את הבית הקטן והקהילתי שבנית בבקעה.
-פרקו היא אפליקציה אחת לכרטיסי מועדון של עסקים בשכונה. הלקוח סורק קוד בקופה וצובר חותמות לפי מה שתבחרי, למשל קנקן תה או סקונס במתנה, וגם קנייה של תה לבית יכולה להיספר.
-אנחנו רוצים לחזק את העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כרגע אנחנו בגישה מוקדמת, וההצטרפות בחינם ובלי התחייבות.
+כאן [השם שלך] מפרקו. קראנו על קומקום ואהבנו את הבית הקטן והקהילתי שבנית בבקעה, עם תה של אחר הצהריים, סקונס ביתיים ופינה של תה עלים.
+פרקו היא אפליקציה אחת לכרטיסי מועדון של עסקים שכונתיים. במקום כרטיס נייר, הלקוח סורק קוד בקופה, צובר חותמות לפי הכללים שאת קובעת, ורואה באותה אפליקציה גם עסקים שכנים בדרך בית לחם.
+מה זה יכול לתת לקומקום:
+- הטבה עם אופי, למשל קנקן תה או סקונס במתנה.
+- גם קנייה של תה עלים לבית יכולה להיספר, כך שהכרטיס עובד גם בין ביקור לביקור.
+- חשיפה ללקוחות של בתי הקפה ברחוב שעוד לא גילו את הגינה שלך.
+אנחנו בשלב גישה מוקדמת ומחפשים כמה עסקים ראשונים בדרך בית לחם שיעזרו לנו לבנות את זה נכון. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום, ונעזור לך בהקמה. המטרה שלנו פשוטה: לחזק את העסקים הקטנים והמשפחתיים שעושים את השכונה לבית.
 אשמח לבוא לתה ולהראות את זה בכמה דקות. מתי נוח לך?
-[השם שלך]</t>
+תודה,
+[השם שלך]
+פרקו · getperko.com</t>
         </is>
       </c>
     </row>
@@ -2560,12 +2644,17 @@
       <c r="X19" s="9" t="inlineStr">
         <is>
           <t>שלום לצוות פוקצ'ה במושבה,
-כאן [השם שלך] מפרקו. שוק הפוקצ'ות שלכם בשישי הוא בדיוק הרגל שבועי ששווה לתגמל.
-פרקו היא אפליקציה אחת לכרטיסי מועדון של עסקים בשכונה. הלקוח סורק קוד בקופה וצובר חותמות לפי הכללים שלכם, למשל פוקצ'ה עליכם בשישי העשירי.
-אנחנו רוצים לחזק את העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כרגע אנחנו בגישה מוקדמת, וההצטרפות בחינם ובלי התחייבות.
+כאן [השם שלך] מפרקו. שוק הפוקצ'ות שלכם בשישי לפני שבת הוא בדיוק הרגל שבועי ששווה לתגמל.
+פרקו היא אפליקציה אחת לכרטיסי מועדון של עסקים שכונתיים. במקום כרטיס נייר, הלקוח סורק קוד בקופה, צובר חותמות לפי הכללים שאתם קובעים, ורואה באותה אפליקציה גם עסקים שכנים בעמק רפאים.
+מה זה יכול לתת לפוקצ'ה במושבה:
+- הטבה שמחזקת את האיסוף של שישי, למשל פוקצ'ה עליכם בשישי העשירי.
+- הלקוח רואה בטלפון כמה חסר לו, ויש סיבה לא לפספס שבוע.
+- הנוכחות שלכם ברחוב עוזרת לרשת, והרשת מביאה לכם לקוחות של העסקים השכנים.
+אנחנו בשלב גישה מוקדמת ומחפשים כמה עסקים ראשונים בעמק רפאים שיעזרו לנו לבנות את זה נכון. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום, ונעזור אתכם בהקמה. המטרה שלנו פשוטה: לחזק את העסקים הקטנים והמשפחתיים שעושים את השכונה לבית.
 אשמח לדבר עם מי שמנהל את המקום. מתי נוח?
 תודה,
-[השם שלך]</t>
+[השם שלך]
+פרקו · getperko.com</t>
         </is>
       </c>
     </row>
@@ -2662,12 +2751,17 @@
       <c r="X20" s="5" t="inlineStr">
         <is>
           <t>שלום לצוות פומפידו,
-כאן [השם שלך] מפרקו. אנחנו בונים אפליקציה אחת לכרטיסי מועדון של עסקים בעמק רפאים, וחשבנו עליכם בגלל החיבור לשכנים ברחוב.
-לקוחות שמכירים את הרחוב מבתי הקפה ביום יכולים לגלות אתכם בערב דרך אותה אפליקציה. הם סורקים קוד בקופה וצוברים נקודות לפי ההטבה שאתם קובעים, למשל קינוח עליכם בביקור הרביעי.
-אנחנו רוצים לחזק את העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כרגע אנחנו בגישה מוקדמת, וההצטרפות בחינם ובלי התחייבות.
+כאן [השם שלך] מפרקו. חשבנו עליכם בגלל החיבור לשכנים: לקוחות שמכירים את עמק רפאים מבתי הקפה ביום יכולים לגלות את הביסטרו והמרפסת שלכם בערב.
+פרקו היא אפליקציה אחת לכרטיסי מועדון של עסקים שכונתיים. במקום כרטיס נייר, הלקוח סורק קוד בקופה, צובר חותמות או נקודות לפי ההטבה שאתם קובעים, ורואה באותה אפליקציה גם עסקים שכנים בעמק רפאים.
+מה זה יכול לתת לפומפידו:
+- חשיפה ללקוחות של העסקים השכנים באותה אפליקציה.
+- הטבה שמחזירה סועדים שלא הגיעו מזמן, למשל קינוח עליכם בביקור הרביעי.
+- בלי קופונים מודפסים ובלי מערכת חדשה במשמרת.
+אנחנו בשלב גישה מוקדמת ומחפשים כמה עסקים ראשונים בעמק רפאים שיעזרו לנו לבנות את זה נכון. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום, ונעזור אתכם בהקמה. המטרה שלנו פשוטה: לחזק את העסקים הקטנים והמשפחתיים שעושים את השכונה לבית.
 אשמח לדבר עם מי שמנהל את המקום. מתי אפשר לתפוס אתכם?
 תודה,
-[השם שלך]</t>
+[השם שלך]
+פרקו · getperko.com</t>
         </is>
       </c>
     </row>
@@ -2764,11 +2858,17 @@
       <c r="X21" s="9" t="inlineStr">
         <is>
           <t>שלום לצוות רנדבו,
-כאן [השם שלך] מפרקו. פיצה ופסטה הן הזמנות שמשפחות חוזרות אליהן שוב ושוב, ושם כרטיס חותמות עובד הכי טוב.
-פרקו היא אפליקציה אחת לכרטיסי מועדון של עסקים בשכונה. הלקוח סורק קוד בקופה וצובר חותמות לפי הכללים שלכם, ורואה שם גם עסקים נוספים בדרך בית לחם.
-אנחנו רוצים לחזק את העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כרגע אנחנו בגישה מוקדמת, וההצטרפות בחינם ובלי התחייבות.
+כאן [השם שלך] מפרקו. פיצה ופסטה הן הזמנות שמשפחות חוזרות אליהן שוב ושוב, וזה בדיוק המקום שבו כרטיס חותמות עובד הכי טוב.
+פרקו היא אפליקציה אחת לכרטיסי מועדון של עסקים שכונתיים. במקום כרטיס נייר, הלקוח סורק קוד בקופה, צובר חותמות לפי הכללים שאתם קובעים, ורואה באותה אפליקציה גם עסקים שכנים בדרך בית לחם.
+מה זה יכול לתת לרנדבו:
+- הטבה משפחתית פשוטה, למשל פיצה במתנה אחרי כמה ביקורים.
+- קשר עם הלקוחות הקבועים, בלי אפליקציה נפרדת.
+- אתם בקצה הדרומי של הרחוב, ותוכלו להביא לרשת לקוחות מכיוון תלפיות.
+אנחנו בשלב גישה מוקדמת ומחפשים כמה עסקים ראשונים בדרך בית לחם שיעזרו לנו לבנות את זה נכון. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום, ונעזור אתכם בהקמה. המטרה שלנו פשוטה: לחזק את העסקים הקטנים והמשפחתיים שעושים את השכונה לבית.
 אשמח לשיחה קצרה עם מי שמנהל את המקום. מתי נוח?
-[השם שלך]</t>
+תודה,
+[השם שלך]
+פרקו · getperko.com</t>
         </is>
       </c>
     </row>
@@ -2873,12 +2973,17 @@
       <c r="X22" s="5" t="inlineStr">
         <is>
           <t>שלום ברברה,
-כאן [השם שלך] מפרקו. אנחנו בונים אפליקציה אחת לכרטיסי מועדון של עסקים בעמק רפאים, וחשבנו על החנות שלך.
-בשביל חנות מתנות היתרון הוא החשיפה: לקוחות קבועים של בתי הקפה והמאפיות ברחוב יכולים לגלות אותך, במיוחד לפני החגים. ההטבה יכולה להיות קטנה, כמו עטיפת מתנה או הנחה לקנייה הבאה.
-אנחנו רוצים לחזק את העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כרגע אנחנו בגישה מוקדמת, וההצטרפות בחינם ובלי התחייבות.
+כאן [השם שלך] מפרקו. החנות שלך יושבת בתחילת עמק רפאים, בדיוק איפה שאנשים מתחילים ללכת ברחוב, עם מתנות שמיוצרות כאן בירושלים.
+פרקו היא אפליקציה אחת לכרטיסי מועדון של עסקים שכונתיים. הלקוח סורק קוד בקופה, צובר הטבות לפי הכללים של כל עסק, ורואה באותה אפליקציה את כל העסקים המשתתפים ברחוב.
+מה זה יכול לתת לברברה שו:
+- חשיפה ללקוחות הקבועים של בתי הקפה והמאפיות ברחוב, במיוחד לפני החגים.
+- הטבה קטנה עם אופי, כמו עטיפת מתנה או הנחה לקנייה הבאה.
+- סיבה לחזור לחנות גם בין עונה לעונה.
+אנחנו בשלב גישה מוקדמת ומחפשים כמה עסקים ראשונים בעמק רפאים שיעזרו לנו לבנות את זה נכון. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום, ונעזור לך בהקמה. המטרה שלנו פשוטה: לחזק את העסקים הקטנים והמשפחתיים שעושים את השכונה לבית.
 אשמח לשמוע אם זה מעניין אותך.
 תודה,
-[השם שלך]</t>
+[השם שלך]
+פרקו · getperko.com</t>
         </is>
       </c>
     </row>
@@ -3000,11 +3105,16 @@
         <is>
           <t>שלום דליה ואייל,
 כאן [השם שלך] מפרקו. סתיו תכשיטים הוא מהעסקים הוותיקים והמיוחדים בעמק רפאים, בדיוק מהמקומות שאנחנו רוצים שאנשים מהשכונה יגלו.
-פרקו היא אפליקציה אחת לכרטיסי מועדון של עסקים ברחוב. אצלכם זה לא חייב להיות כרטיס חותמות רגיל: אפשר להגדיר הטבה שמתאימה לתכשיטים, כמו ניקוי, תיקון או חריטה במתנה.
-אנחנו רוצים לחזק את העסקים הקטנים והמשפחתיים שעושים את השכונה לבית. כרגע אנחנו בגישה מוקדמת, וההצטרפות בחינם ובלי התחייבות.
+פרקו היא אפליקציה אחת לכרטיסי מועדון של עסקים שכונתיים. במקום כרטיס נייר, הלקוח סורק קוד בקופה, צובר חותמות או הטבות לפי הכללים שאתם קובעים, ורואה באותה אפליקציה גם עסקים שכנים בעמק רפאים.
+מה זה יכול לתת לסתיו תכשיטים:
+- הטבה שמתאימה לתכשיטים ולא לקפה, כמו ניקוי, תיקון או חריטה במתנה.
+- חשיפה ללקוחות הקבועים של בתי הקפה והמאפיות ברחוב, שמחפשים מתנה מקומית.
+- קשר שנשאר עם הלקוח גם אחרי הקנייה, לקראת החג הבא.
+אנחנו בשלב גישה מוקדמת ומחפשים כמה עסקים ראשונים בעמק רפאים שיעזרו לנו לבנות את זה נכון. ההצטרפות כרגע בחינם ובלי התחייבות לתשלום, ונעזור אתכם בהקמה. המטרה שלנו פשוטה: לחזק את העסקים הקטנים והמשפחתיים שעושים את השכונה לבית.
 אשמח לשמוע אם זה מעניין אתכם, ולקפוץ לשיחה קצרה.
 תודה,
-[השם שלך]</t>
+[השם שלך]
+פרקו · getperko.com</t>
         </is>
       </c>
     </row>

</xml_diff>